<commit_message>
Regenerate tax PDFs + ZIPs with AllPro Construction & Landscape name
Co-authored-by: Copilot <223556219+Copilot@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/bill-docs-k7m2v9/AllPro_Tax_2025.xlsx
+++ b/bill-docs-k7m2v9/AllPro_Tax_2025.xlsx
@@ -493,6 +493,7 @@
         <v>20676.13</v>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
@@ -510,6 +511,7 @@
         <v>49194.49</v>
       </c>
     </row>
+    <row r="5"/>
     <row r="6">
       <c r="A6" s="1" t="inlineStr">
         <is>
@@ -11422,7 +11424,6 @@
         <f>IF(G2&lt;&gt;F2,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="5" t="n">
@@ -11459,7 +11460,6 @@
         <f>IF(G3&lt;&gt;F3,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="5" t="n">
@@ -11496,7 +11496,6 @@
         <f>IF(G4&lt;&gt;F4,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="5" t="n">
@@ -11533,7 +11532,6 @@
         <f>IF(G5&lt;&gt;F5,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="5" t="n">
@@ -11570,7 +11568,6 @@
         <f>IF(G6&lt;&gt;F6,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="5" t="n">
@@ -11607,7 +11604,6 @@
         <f>IF(G7&lt;&gt;F7,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="5" t="n">
@@ -11644,7 +11640,6 @@
         <f>IF(G8&lt;&gt;F8,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="5" t="n">
@@ -11681,7 +11676,6 @@
         <f>IF(G9&lt;&gt;F9,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="5" t="n">
@@ -11718,7 +11712,6 @@
         <f>IF(G10&lt;&gt;F10,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="5" t="n">
@@ -11755,7 +11748,6 @@
         <f>IF(G11&lt;&gt;F11,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="5" t="n">
@@ -11792,7 +11784,6 @@
         <f>IF(G12&lt;&gt;F12,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="5" t="n">
@@ -11829,7 +11820,6 @@
         <f>IF(G13&lt;&gt;F13,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="5" t="n">
@@ -11866,7 +11856,6 @@
         <f>IF(G14&lt;&gt;F14,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="5" t="n">
@@ -11903,7 +11892,6 @@
         <f>IF(G15&lt;&gt;F15,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="5" t="n">
@@ -11940,7 +11928,6 @@
         <f>IF(G16&lt;&gt;F16,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="5" t="n">
@@ -11977,7 +11964,6 @@
         <f>IF(G17&lt;&gt;F17,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="5" t="n">
@@ -12014,7 +12000,6 @@
         <f>IF(G18&lt;&gt;F18,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="5" t="n">
@@ -12051,7 +12036,6 @@
         <f>IF(G19&lt;&gt;F19,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="5" t="n">
@@ -12088,7 +12072,6 @@
         <f>IF(G20&lt;&gt;F20,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="5" t="n">
@@ -12125,7 +12108,6 @@
         <f>IF(G21&lt;&gt;F21,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="5" t="n">
@@ -12162,7 +12144,6 @@
         <f>IF(G22&lt;&gt;F22,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="5" t="n">
@@ -12199,7 +12180,6 @@
         <f>IF(G23&lt;&gt;F23,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="5" t="n">
@@ -12236,7 +12216,6 @@
         <f>IF(G24&lt;&gt;F24,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="5" t="n">
@@ -12273,7 +12252,6 @@
         <f>IF(G25&lt;&gt;F25,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="5" t="n">
@@ -12310,7 +12288,6 @@
         <f>IF(G26&lt;&gt;F26,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="5" t="n">
@@ -12347,7 +12324,6 @@
         <f>IF(G27&lt;&gt;F27,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="5" t="n">
@@ -12384,7 +12360,6 @@
         <f>IF(G28&lt;&gt;F28,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" s="5" t="n">
@@ -12421,7 +12396,6 @@
         <f>IF(G29&lt;&gt;F29,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" s="5" t="n">
@@ -12458,7 +12432,6 @@
         <f>IF(G30&lt;&gt;F30,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" s="5" t="n">
@@ -12495,7 +12468,6 @@
         <f>IF(G31&lt;&gt;F31,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" s="5" t="n">
@@ -12532,7 +12504,6 @@
         <f>IF(G32&lt;&gt;F32,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" s="5" t="n">
@@ -12569,7 +12540,6 @@
         <f>IF(G33&lt;&gt;F33,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" s="5" t="n">
@@ -12606,7 +12576,6 @@
         <f>IF(G34&lt;&gt;F34,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" s="5" t="n">
@@ -12643,7 +12612,6 @@
         <f>IF(G35&lt;&gt;F35,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" s="5" t="n">
@@ -12680,7 +12648,6 @@
         <f>IF(G36&lt;&gt;F36,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" s="5" t="n">
@@ -12717,7 +12684,6 @@
         <f>IF(G37&lt;&gt;F37,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" s="5" t="n">
@@ -12754,7 +12720,6 @@
         <f>IF(G38&lt;&gt;F38,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" s="5" t="n">
@@ -12791,7 +12756,6 @@
         <f>IF(G39&lt;&gt;F39,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" s="5" t="n">
@@ -12828,7 +12792,6 @@
         <f>IF(G40&lt;&gt;F40,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" s="5" t="n">
@@ -12865,7 +12828,6 @@
         <f>IF(G41&lt;&gt;F41,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" s="5" t="n">
@@ -12902,7 +12864,6 @@
         <f>IF(G42&lt;&gt;F42,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" s="5" t="n">
@@ -12939,7 +12900,6 @@
         <f>IF(G43&lt;&gt;F43,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" s="5" t="n">
@@ -12976,7 +12936,6 @@
         <f>IF(G44&lt;&gt;F44,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" s="5" t="n">
@@ -13013,7 +12972,6 @@
         <f>IF(G45&lt;&gt;F45,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" s="5" t="n">
@@ -13050,7 +13008,6 @@
         <f>IF(G46&lt;&gt;F46,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" s="5" t="n">
@@ -13087,7 +13044,6 @@
         <f>IF(G47&lt;&gt;F47,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" s="5" t="n">
@@ -13124,7 +13080,6 @@
         <f>IF(G48&lt;&gt;F48,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" s="5" t="n">
@@ -13161,7 +13116,6 @@
         <f>IF(G49&lt;&gt;F49,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" s="5" t="n">
@@ -13198,7 +13152,6 @@
         <f>IF(G50&lt;&gt;F50,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" s="5" t="n">
@@ -13235,7 +13188,6 @@
         <f>IF(G51&lt;&gt;F51,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" s="5" t="n">
@@ -13272,7 +13224,6 @@
         <f>IF(G52&lt;&gt;F52,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" s="5" t="n">
@@ -13309,7 +13260,6 @@
         <f>IF(G53&lt;&gt;F53,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" s="5" t="n">
@@ -13346,7 +13296,6 @@
         <f>IF(G54&lt;&gt;F54,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" s="5" t="n">
@@ -13383,7 +13332,6 @@
         <f>IF(G55&lt;&gt;F55,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" s="5" t="n">
@@ -13420,7 +13368,6 @@
         <f>IF(G56&lt;&gt;F56,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" s="5" t="n">
@@ -13457,7 +13404,6 @@
         <f>IF(G57&lt;&gt;F57,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" s="5" t="n">
@@ -13494,7 +13440,6 @@
         <f>IF(G58&lt;&gt;F58,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" s="5" t="n">
@@ -13531,7 +13476,6 @@
         <f>IF(G59&lt;&gt;F59,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" s="5" t="n">
@@ -13568,7 +13512,6 @@
         <f>IF(G60&lt;&gt;F60,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I60" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" s="5" t="n">
@@ -13605,7 +13548,6 @@
         <f>IF(G61&lt;&gt;F61,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I61" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" s="5" t="n">
@@ -13642,7 +13584,6 @@
         <f>IF(G62&lt;&gt;F62,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I62" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" s="5" t="n">
@@ -13679,7 +13620,6 @@
         <f>IF(G63&lt;&gt;F63,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I63" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" s="5" t="n">
@@ -13716,7 +13656,6 @@
         <f>IF(G64&lt;&gt;F64,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I64" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" s="5" t="n">
@@ -13753,7 +13692,6 @@
         <f>IF(G65&lt;&gt;F65,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I65" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" s="5" t="n">
@@ -13790,7 +13728,6 @@
         <f>IF(G66&lt;&gt;F66,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I66" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" s="5" t="n">
@@ -13827,7 +13764,6 @@
         <f>IF(G67&lt;&gt;F67,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I67" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" s="5" t="n">
@@ -13864,7 +13800,6 @@
         <f>IF(G68&lt;&gt;F68,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I68" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" s="5" t="n">
@@ -13901,7 +13836,6 @@
         <f>IF(G69&lt;&gt;F69,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I69" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" s="5" t="n">
@@ -13938,7 +13872,6 @@
         <f>IF(G70&lt;&gt;F70,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I70" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" s="5" t="n">
@@ -13975,7 +13908,6 @@
         <f>IF(G71&lt;&gt;F71,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I71" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" s="5" t="n">
@@ -14012,7 +13944,6 @@
         <f>IF(G72&lt;&gt;F72,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I72" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" s="5" t="n">
@@ -14049,7 +13980,6 @@
         <f>IF(G73&lt;&gt;F73,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I73" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" s="5" t="n">
@@ -14086,7 +14016,6 @@
         <f>IF(G74&lt;&gt;F74,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I74" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" s="5" t="n">
@@ -14123,7 +14052,6 @@
         <f>IF(G75&lt;&gt;F75,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I75" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" s="5" t="n">
@@ -14160,7 +14088,6 @@
         <f>IF(G76&lt;&gt;F76,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I76" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" s="5" t="n">
@@ -14197,7 +14124,6 @@
         <f>IF(G77&lt;&gt;F77,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I77" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" s="5" t="n">
@@ -14234,7 +14160,6 @@
         <f>IF(G78&lt;&gt;F78,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I78" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" s="5" t="n">
@@ -14271,7 +14196,6 @@
         <f>IF(G79&lt;&gt;F79,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I79" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" s="5" t="n">
@@ -14308,7 +14232,6 @@
         <f>IF(G80&lt;&gt;F80,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I80" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" s="5" t="n">
@@ -14345,7 +14268,6 @@
         <f>IF(G81&lt;&gt;F81,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I81" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" s="5" t="n">
@@ -14382,7 +14304,6 @@
         <f>IF(G82&lt;&gt;F82,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I82" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" s="5" t="n">
@@ -14419,7 +14340,6 @@
         <f>IF(G83&lt;&gt;F83,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I83" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" s="5" t="n">
@@ -14456,7 +14376,6 @@
         <f>IF(G84&lt;&gt;F84,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I84" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" s="5" t="n">
@@ -14493,7 +14412,6 @@
         <f>IF(G85&lt;&gt;F85,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I85" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" s="5" t="n">
@@ -14530,7 +14448,6 @@
         <f>IF(G86&lt;&gt;F86,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I86" t="inlineStr"/>
     </row>
     <row r="87">
       <c r="A87" s="5" t="n">
@@ -14567,7 +14484,6 @@
         <f>IF(G87&lt;&gt;F87,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I87" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" s="5" t="n">
@@ -14604,7 +14520,6 @@
         <f>IF(G88&lt;&gt;F88,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I88" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" s="5" t="n">
@@ -14641,7 +14556,6 @@
         <f>IF(G89&lt;&gt;F89,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I89" t="inlineStr"/>
     </row>
     <row r="90">
       <c r="A90" s="5" t="n">
@@ -14678,7 +14592,6 @@
         <f>IF(G90&lt;&gt;F90,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I90" t="inlineStr"/>
     </row>
     <row r="91">
       <c r="A91" s="5" t="n">
@@ -14715,7 +14628,6 @@
         <f>IF(G91&lt;&gt;F91,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I91" t="inlineStr"/>
     </row>
     <row r="92">
       <c r="A92" s="5" t="n">
@@ -14752,7 +14664,6 @@
         <f>IF(G92&lt;&gt;F92,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I92" t="inlineStr"/>
     </row>
     <row r="93">
       <c r="A93" s="5" t="n">
@@ -14789,7 +14700,6 @@
         <f>IF(G93&lt;&gt;F93,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I93" t="inlineStr"/>
     </row>
     <row r="94">
       <c r="A94" s="5" t="n">
@@ -14826,7 +14736,6 @@
         <f>IF(G94&lt;&gt;F94,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I94" t="inlineStr"/>
     </row>
     <row r="95">
       <c r="A95" s="5" t="n">
@@ -14863,7 +14772,6 @@
         <f>IF(G95&lt;&gt;F95,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I95" t="inlineStr"/>
     </row>
     <row r="96">
       <c r="A96" s="5" t="n">
@@ -14900,7 +14808,6 @@
         <f>IF(G96&lt;&gt;F96,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I96" t="inlineStr"/>
     </row>
     <row r="97">
       <c r="A97" s="5" t="n">
@@ -14937,7 +14844,6 @@
         <f>IF(G97&lt;&gt;F97,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I97" t="inlineStr"/>
     </row>
     <row r="98">
       <c r="A98" s="5" t="n">
@@ -14974,7 +14880,6 @@
         <f>IF(G98&lt;&gt;F98,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I98" t="inlineStr"/>
     </row>
     <row r="99">
       <c r="A99" s="5" t="n">
@@ -15011,7 +14916,6 @@
         <f>IF(G99&lt;&gt;F99,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I99" t="inlineStr"/>
     </row>
     <row r="100">
       <c r="A100" s="5" t="n">
@@ -15048,7 +14952,6 @@
         <f>IF(G100&lt;&gt;F100,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I100" t="inlineStr"/>
     </row>
     <row r="101">
       <c r="A101" s="5" t="n">
@@ -15085,7 +14988,6 @@
         <f>IF(G101&lt;&gt;F101,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I101" t="inlineStr"/>
     </row>
     <row r="102">
       <c r="A102" s="5" t="n">
@@ -15122,7 +15024,6 @@
         <f>IF(G102&lt;&gt;F102,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I102" t="inlineStr"/>
     </row>
     <row r="103">
       <c r="A103" s="5" t="n">
@@ -15159,7 +15060,6 @@
         <f>IF(G103&lt;&gt;F103,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I103" t="inlineStr"/>
     </row>
     <row r="104">
       <c r="A104" s="5" t="n">
@@ -15196,7 +15096,6 @@
         <f>IF(G104&lt;&gt;F104,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I104" t="inlineStr"/>
     </row>
     <row r="105">
       <c r="A105" s="5" t="n">
@@ -15233,7 +15132,6 @@
         <f>IF(G105&lt;&gt;F105,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I105" t="inlineStr"/>
     </row>
     <row r="106">
       <c r="A106" s="5" t="n">
@@ -15270,7 +15168,6 @@
         <f>IF(G106&lt;&gt;F106,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I106" t="inlineStr"/>
     </row>
     <row r="107">
       <c r="A107" s="5" t="n">
@@ -15307,7 +15204,6 @@
         <f>IF(G107&lt;&gt;F107,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I107" t="inlineStr"/>
     </row>
     <row r="108">
       <c r="A108" s="5" t="n">
@@ -15344,7 +15240,6 @@
         <f>IF(G108&lt;&gt;F108,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I108" t="inlineStr"/>
     </row>
     <row r="109">
       <c r="A109" s="5" t="n">
@@ -15381,7 +15276,6 @@
         <f>IF(G109&lt;&gt;F109,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I109" t="inlineStr"/>
     </row>
     <row r="110">
       <c r="A110" s="5" t="n">
@@ -15418,7 +15312,6 @@
         <f>IF(G110&lt;&gt;F110,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I110" t="inlineStr"/>
     </row>
     <row r="111">
       <c r="A111" s="5" t="n">
@@ -15455,7 +15348,6 @@
         <f>IF(G111&lt;&gt;F111,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I111" t="inlineStr"/>
     </row>
     <row r="112">
       <c r="A112" s="5" t="n">
@@ -15492,7 +15384,6 @@
         <f>IF(G112&lt;&gt;F112,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I112" t="inlineStr"/>
     </row>
     <row r="113">
       <c r="A113" s="5" t="n">
@@ -15529,7 +15420,6 @@
         <f>IF(G113&lt;&gt;F113,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I113" t="inlineStr"/>
     </row>
     <row r="114">
       <c r="A114" s="5" t="n">
@@ -15566,7 +15456,6 @@
         <f>IF(G114&lt;&gt;F114,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I114" t="inlineStr"/>
     </row>
     <row r="115">
       <c r="A115" s="5" t="n">
@@ -15603,7 +15492,6 @@
         <f>IF(G115&lt;&gt;F115,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I115" t="inlineStr"/>
     </row>
     <row r="116">
       <c r="A116" s="5" t="n">
@@ -15640,7 +15528,6 @@
         <f>IF(G116&lt;&gt;F116,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I116" t="inlineStr"/>
     </row>
     <row r="117">
       <c r="A117" s="5" t="n">
@@ -15677,7 +15564,6 @@
         <f>IF(G117&lt;&gt;F117,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I117" t="inlineStr"/>
     </row>
     <row r="118">
       <c r="A118" s="5" t="n">
@@ -15714,7 +15600,6 @@
         <f>IF(G118&lt;&gt;F118,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I118" t="inlineStr"/>
     </row>
     <row r="119">
       <c r="A119" s="5" t="n">
@@ -15751,7 +15636,6 @@
         <f>IF(G119&lt;&gt;F119,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I119" t="inlineStr"/>
     </row>
     <row r="120">
       <c r="A120" s="5" t="n">
@@ -15788,7 +15672,6 @@
         <f>IF(G120&lt;&gt;F120,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I120" t="inlineStr"/>
     </row>
     <row r="121">
       <c r="A121" s="5" t="n">
@@ -15825,7 +15708,6 @@
         <f>IF(G121&lt;&gt;F121,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I121" t="inlineStr"/>
     </row>
     <row r="122">
       <c r="A122" s="5" t="n">
@@ -15862,7 +15744,6 @@
         <f>IF(G122&lt;&gt;F122,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I122" t="inlineStr"/>
     </row>
     <row r="123">
       <c r="A123" s="5" t="n">
@@ -15899,7 +15780,6 @@
         <f>IF(G123&lt;&gt;F123,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I123" t="inlineStr"/>
     </row>
     <row r="124">
       <c r="A124" s="5" t="n">
@@ -15936,7 +15816,6 @@
         <f>IF(G124&lt;&gt;F124,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I124" t="inlineStr"/>
     </row>
     <row r="125">
       <c r="A125" s="5" t="n">
@@ -15973,7 +15852,6 @@
         <f>IF(G125&lt;&gt;F125,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I125" t="inlineStr"/>
     </row>
     <row r="126">
       <c r="A126" s="5" t="n">
@@ -16010,7 +15888,6 @@
         <f>IF(G126&lt;&gt;F126,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I126" t="inlineStr"/>
     </row>
     <row r="127">
       <c r="A127" s="5" t="n">
@@ -16047,7 +15924,6 @@
         <f>IF(G127&lt;&gt;F127,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I127" t="inlineStr"/>
     </row>
     <row r="128">
       <c r="A128" s="5" t="n">
@@ -16084,7 +15960,6 @@
         <f>IF(G128&lt;&gt;F128,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I128" t="inlineStr"/>
     </row>
     <row r="129">
       <c r="A129" s="5" t="n">
@@ -16121,7 +15996,6 @@
         <f>IF(G129&lt;&gt;F129,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I129" t="inlineStr"/>
     </row>
     <row r="130">
       <c r="A130" s="5" t="n">
@@ -16158,7 +16032,6 @@
         <f>IF(G130&lt;&gt;F130,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I130" t="inlineStr"/>
     </row>
     <row r="131">
       <c r="A131" s="5" t="n">
@@ -16195,7 +16068,6 @@
         <f>IF(G131&lt;&gt;F131,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I131" t="inlineStr"/>
     </row>
     <row r="132">
       <c r="A132" s="5" t="n">
@@ -16232,7 +16104,6 @@
         <f>IF(G132&lt;&gt;F132,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I132" t="inlineStr"/>
     </row>
     <row r="133">
       <c r="A133" s="5" t="n">
@@ -16269,7 +16140,6 @@
         <f>IF(G133&lt;&gt;F133,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I133" t="inlineStr"/>
     </row>
     <row r="134">
       <c r="A134" s="5" t="n">
@@ -16306,7 +16176,6 @@
         <f>IF(G134&lt;&gt;F134,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I134" t="inlineStr"/>
     </row>
     <row r="135">
       <c r="A135" s="5" t="n">
@@ -16343,7 +16212,6 @@
         <f>IF(G135&lt;&gt;F135,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I135" t="inlineStr"/>
     </row>
     <row r="136">
       <c r="A136" s="5" t="n">
@@ -16380,7 +16248,6 @@
         <f>IF(G136&lt;&gt;F136,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I136" t="inlineStr"/>
     </row>
     <row r="137">
       <c r="A137" s="5" t="n">
@@ -16417,7 +16284,6 @@
         <f>IF(G137&lt;&gt;F137,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I137" t="inlineStr"/>
     </row>
     <row r="138">
       <c r="A138" s="5" t="n">
@@ -16454,7 +16320,6 @@
         <f>IF(G138&lt;&gt;F138,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I138" t="inlineStr"/>
     </row>
     <row r="139">
       <c r="A139" s="5" t="n">
@@ -16491,7 +16356,6 @@
         <f>IF(G139&lt;&gt;F139,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I139" t="inlineStr"/>
     </row>
     <row r="140">
       <c r="A140" s="5" t="n">
@@ -16528,7 +16392,6 @@
         <f>IF(G140&lt;&gt;F140,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I140" t="inlineStr"/>
     </row>
     <row r="141">
       <c r="A141" s="5" t="n">
@@ -16565,7 +16428,6 @@
         <f>IF(G141&lt;&gt;F141,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I141" t="inlineStr"/>
     </row>
     <row r="142">
       <c r="A142" s="5" t="n">
@@ -16602,7 +16464,6 @@
         <f>IF(G142&lt;&gt;F142,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I142" t="inlineStr"/>
     </row>
     <row r="143">
       <c r="A143" s="5" t="n">
@@ -16639,7 +16500,6 @@
         <f>IF(G143&lt;&gt;F143,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I143" t="inlineStr"/>
     </row>
     <row r="144">
       <c r="A144" s="5" t="n">
@@ -16676,7 +16536,6 @@
         <f>IF(G144&lt;&gt;F144,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I144" t="inlineStr"/>
     </row>
     <row r="145">
       <c r="A145" s="5" t="n">
@@ -16713,7 +16572,6 @@
         <f>IF(G145&lt;&gt;F145,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I145" t="inlineStr"/>
     </row>
     <row r="146">
       <c r="A146" s="5" t="n">
@@ -16750,7 +16608,6 @@
         <f>IF(G146&lt;&gt;F146,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I146" t="inlineStr"/>
     </row>
     <row r="147">
       <c r="A147" s="5" t="n">
@@ -16787,7 +16644,6 @@
         <f>IF(G147&lt;&gt;F147,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I147" t="inlineStr"/>
     </row>
     <row r="148">
       <c r="A148" s="5" t="n">
@@ -16824,7 +16680,6 @@
         <f>IF(G148&lt;&gt;F148,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I148" t="inlineStr"/>
     </row>
     <row r="149">
       <c r="A149" s="5" t="n">
@@ -16861,7 +16716,6 @@
         <f>IF(G149&lt;&gt;F149,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I149" t="inlineStr"/>
     </row>
     <row r="150">
       <c r="A150" s="5" t="n">
@@ -16898,7 +16752,6 @@
         <f>IF(G150&lt;&gt;F150,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I150" t="inlineStr"/>
     </row>
     <row r="151">
       <c r="A151" s="5" t="n">
@@ -16935,7 +16788,6 @@
         <f>IF(G151&lt;&gt;F151,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I151" t="inlineStr"/>
     </row>
     <row r="152">
       <c r="A152" s="5" t="n">
@@ -16972,7 +16824,6 @@
         <f>IF(G152&lt;&gt;F152,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I152" t="inlineStr"/>
     </row>
     <row r="153">
       <c r="A153" s="5" t="n">
@@ -17009,7 +16860,6 @@
         <f>IF(G153&lt;&gt;F153,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I153" t="inlineStr"/>
     </row>
     <row r="154">
       <c r="A154" s="5" t="n">
@@ -17046,7 +16896,6 @@
         <f>IF(G154&lt;&gt;F154,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I154" t="inlineStr"/>
     </row>
     <row r="155">
       <c r="A155" s="5" t="n">
@@ -17083,7 +16932,6 @@
         <f>IF(G155&lt;&gt;F155,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I155" t="inlineStr"/>
     </row>
     <row r="156">
       <c r="A156" s="5" t="n">
@@ -17120,7 +16968,6 @@
         <f>IF(G156&lt;&gt;F156,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I156" t="inlineStr"/>
     </row>
     <row r="157">
       <c r="A157" s="5" t="n">
@@ -17157,7 +17004,6 @@
         <f>IF(G157&lt;&gt;F157,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I157" t="inlineStr"/>
     </row>
     <row r="158">
       <c r="A158" s="5" t="n">
@@ -17194,7 +17040,6 @@
         <f>IF(G158&lt;&gt;F158,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I158" t="inlineStr"/>
     </row>
     <row r="159">
       <c r="A159" s="5" t="n">
@@ -17231,7 +17076,6 @@
         <f>IF(G159&lt;&gt;F159,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I159" t="inlineStr"/>
     </row>
     <row r="160">
       <c r="A160" s="5" t="n">
@@ -17268,7 +17112,6 @@
         <f>IF(G160&lt;&gt;F160,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I160" t="inlineStr"/>
     </row>
     <row r="161">
       <c r="A161" s="5" t="n">
@@ -17305,7 +17148,6 @@
         <f>IF(G161&lt;&gt;F161,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I161" t="inlineStr"/>
     </row>
     <row r="162">
       <c r="A162" s="5" t="n">
@@ -17342,7 +17184,6 @@
         <f>IF(G162&lt;&gt;F162,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I162" t="inlineStr"/>
     </row>
     <row r="163">
       <c r="A163" s="5" t="n">
@@ -17379,7 +17220,6 @@
         <f>IF(G163&lt;&gt;F163,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I163" t="inlineStr"/>
     </row>
     <row r="164">
       <c r="A164" s="5" t="n">
@@ -17416,7 +17256,6 @@
         <f>IF(G164&lt;&gt;F164,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I164" t="inlineStr"/>
     </row>
     <row r="165">
       <c r="A165" s="5" t="n">
@@ -17453,7 +17292,6 @@
         <f>IF(G165&lt;&gt;F165,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I165" t="inlineStr"/>
     </row>
     <row r="166">
       <c r="A166" s="5" t="n">
@@ -17490,7 +17328,6 @@
         <f>IF(G166&lt;&gt;F166,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I166" t="inlineStr"/>
     </row>
     <row r="167">
       <c r="A167" s="5" t="n">
@@ -17527,7 +17364,6 @@
         <f>IF(G167&lt;&gt;F167,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I167" t="inlineStr"/>
     </row>
     <row r="168">
       <c r="A168" s="5" t="n">
@@ -17564,7 +17400,6 @@
         <f>IF(G168&lt;&gt;F168,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I168" t="inlineStr"/>
     </row>
     <row r="169">
       <c r="A169" s="5" t="n">
@@ -17601,7 +17436,6 @@
         <f>IF(G169&lt;&gt;F169,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I169" t="inlineStr"/>
     </row>
     <row r="170">
       <c r="A170" s="5" t="n">
@@ -17638,7 +17472,6 @@
         <f>IF(G170&lt;&gt;F170,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I170" t="inlineStr"/>
     </row>
     <row r="171">
       <c r="A171" s="5" t="n">
@@ -17675,7 +17508,6 @@
         <f>IF(G171&lt;&gt;F171,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I171" t="inlineStr"/>
     </row>
     <row r="172">
       <c r="A172" s="5" t="n">
@@ -17712,7 +17544,6 @@
         <f>IF(G172&lt;&gt;F172,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I172" t="inlineStr"/>
     </row>
     <row r="173">
       <c r="A173" s="5" t="n">
@@ -17749,7 +17580,6 @@
         <f>IF(G173&lt;&gt;F173,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I173" t="inlineStr"/>
     </row>
     <row r="174">
       <c r="A174" s="5" t="n">
@@ -17786,7 +17616,6 @@
         <f>IF(G174&lt;&gt;F174,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I174" t="inlineStr"/>
     </row>
     <row r="175">
       <c r="A175" s="5" t="n">
@@ -17823,7 +17652,6 @@
         <f>IF(G175&lt;&gt;F175,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I175" t="inlineStr"/>
     </row>
     <row r="176">
       <c r="A176" s="5" t="n">
@@ -17860,7 +17688,6 @@
         <f>IF(G176&lt;&gt;F176,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I176" t="inlineStr"/>
     </row>
     <row r="177">
       <c r="A177" s="5" t="n">
@@ -17897,7 +17724,6 @@
         <f>IF(G177&lt;&gt;F177,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I177" t="inlineStr"/>
     </row>
     <row r="178">
       <c r="A178" s="5" t="n">
@@ -17934,7 +17760,6 @@
         <f>IF(G178&lt;&gt;F178,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I178" t="inlineStr"/>
     </row>
     <row r="179">
       <c r="A179" s="5" t="n">
@@ -17971,7 +17796,6 @@
         <f>IF(G179&lt;&gt;F179,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I179" t="inlineStr"/>
     </row>
     <row r="180">
       <c r="A180" s="5" t="n">
@@ -18008,7 +17832,6 @@
         <f>IF(G180&lt;&gt;F180,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I180" t="inlineStr"/>
     </row>
     <row r="181">
       <c r="A181" s="5" t="n">
@@ -18045,7 +17868,6 @@
         <f>IF(G181&lt;&gt;F181,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I181" t="inlineStr"/>
     </row>
     <row r="182">
       <c r="A182" s="5" t="n">
@@ -18082,7 +17904,6 @@
         <f>IF(G182&lt;&gt;F182,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I182" t="inlineStr"/>
     </row>
     <row r="183">
       <c r="A183" s="5" t="n">
@@ -18119,7 +17940,6 @@
         <f>IF(G183&lt;&gt;F183,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I183" t="inlineStr"/>
     </row>
     <row r="184">
       <c r="A184" s="5" t="n">
@@ -18156,7 +17976,6 @@
         <f>IF(G184&lt;&gt;F184,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I184" t="inlineStr"/>
     </row>
     <row r="185">
       <c r="A185" s="5" t="n">
@@ -18193,7 +18012,6 @@
         <f>IF(G185&lt;&gt;F185,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I185" t="inlineStr"/>
     </row>
     <row r="186">
       <c r="A186" s="5" t="n">
@@ -18230,7 +18048,6 @@
         <f>IF(G186&lt;&gt;F186,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I186" t="inlineStr"/>
     </row>
     <row r="187">
       <c r="A187" s="5" t="n">
@@ -18267,7 +18084,6 @@
         <f>IF(G187&lt;&gt;F187,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I187" t="inlineStr"/>
     </row>
     <row r="188">
       <c r="A188" s="5" t="n">
@@ -18304,7 +18120,6 @@
         <f>IF(G188&lt;&gt;F188,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I188" t="inlineStr"/>
     </row>
     <row r="189">
       <c r="A189" s="5" t="n">
@@ -18341,7 +18156,6 @@
         <f>IF(G189&lt;&gt;F189,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I189" t="inlineStr"/>
     </row>
     <row r="190">
       <c r="A190" s="5" t="n">
@@ -18378,7 +18192,6 @@
         <f>IF(G190&lt;&gt;F190,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I190" t="inlineStr"/>
     </row>
     <row r="191">
       <c r="A191" s="5" t="n">
@@ -18415,7 +18228,6 @@
         <f>IF(G191&lt;&gt;F191,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I191" t="inlineStr"/>
     </row>
     <row r="192">
       <c r="A192" s="5" t="n">
@@ -18452,7 +18264,6 @@
         <f>IF(G192&lt;&gt;F192,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I192" t="inlineStr"/>
     </row>
     <row r="193">
       <c r="A193" s="5" t="n">
@@ -18489,7 +18300,6 @@
         <f>IF(G193&lt;&gt;F193,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I193" t="inlineStr"/>
     </row>
     <row r="194">
       <c r="A194" s="5" t="n">
@@ -18526,7 +18336,6 @@
         <f>IF(G194&lt;&gt;F194,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I194" t="inlineStr"/>
     </row>
     <row r="195">
       <c r="A195" s="5" t="n">
@@ -18563,7 +18372,6 @@
         <f>IF(G195&lt;&gt;F195,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I195" t="inlineStr"/>
     </row>
     <row r="196">
       <c r="A196" s="5" t="n">
@@ -18600,7 +18408,6 @@
         <f>IF(G196&lt;&gt;F196,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I196" t="inlineStr"/>
     </row>
     <row r="197">
       <c r="A197" s="5" t="n">
@@ -18637,7 +18444,6 @@
         <f>IF(G197&lt;&gt;F197,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I197" t="inlineStr"/>
     </row>
     <row r="198">
       <c r="A198" s="5" t="n">
@@ -18674,7 +18480,6 @@
         <f>IF(G198&lt;&gt;F198,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I198" t="inlineStr"/>
     </row>
     <row r="199">
       <c r="A199" s="5" t="n">
@@ -18711,7 +18516,6 @@
         <f>IF(G199&lt;&gt;F199,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I199" t="inlineStr"/>
     </row>
     <row r="200">
       <c r="A200" s="5" t="n">
@@ -18748,7 +18552,6 @@
         <f>IF(G200&lt;&gt;F200,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I200" t="inlineStr"/>
     </row>
     <row r="201">
       <c r="A201" s="5" t="n">
@@ -18785,7 +18588,6 @@
         <f>IF(G201&lt;&gt;F201,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I201" t="inlineStr"/>
     </row>
     <row r="202">
       <c r="A202" s="5" t="n">
@@ -18822,7 +18624,6 @@
         <f>IF(G202&lt;&gt;F202,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I202" t="inlineStr"/>
     </row>
     <row r="203">
       <c r="A203" s="5" t="n">
@@ -18859,7 +18660,6 @@
         <f>IF(G203&lt;&gt;F203,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I203" t="inlineStr"/>
     </row>
     <row r="204">
       <c r="A204" s="5" t="n">
@@ -18896,7 +18696,6 @@
         <f>IF(G204&lt;&gt;F204,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I204" t="inlineStr"/>
     </row>
     <row r="205">
       <c r="A205" s="5" t="n">
@@ -18933,7 +18732,6 @@
         <f>IF(G205&lt;&gt;F205,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I205" t="inlineStr"/>
     </row>
     <row r="206">
       <c r="A206" s="5" t="n">
@@ -18970,7 +18768,6 @@
         <f>IF(G206&lt;&gt;F206,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I206" t="inlineStr"/>
     </row>
     <row r="207">
       <c r="A207" s="5" t="n">
@@ -19007,7 +18804,6 @@
         <f>IF(G207&lt;&gt;F207,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I207" t="inlineStr"/>
     </row>
     <row r="208">
       <c r="A208" s="5" t="n">
@@ -19044,7 +18840,6 @@
         <f>IF(G208&lt;&gt;F208,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I208" t="inlineStr"/>
     </row>
     <row r="209">
       <c r="A209" s="5" t="n">
@@ -19081,7 +18876,6 @@
         <f>IF(G209&lt;&gt;F209,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I209" t="inlineStr"/>
     </row>
     <row r="210">
       <c r="A210" s="5" t="n">
@@ -19118,7 +18912,6 @@
         <f>IF(G210&lt;&gt;F210,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I210" t="inlineStr"/>
     </row>
     <row r="211">
       <c r="A211" s="5" t="n">
@@ -19155,7 +18948,6 @@
         <f>IF(G211&lt;&gt;F211,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I211" t="inlineStr"/>
     </row>
     <row r="212">
       <c r="A212" s="5" t="n">
@@ -19192,7 +18984,6 @@
         <f>IF(G212&lt;&gt;F212,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I212" t="inlineStr"/>
     </row>
     <row r="213">
       <c r="A213" s="5" t="n">
@@ -19229,7 +19020,6 @@
         <f>IF(G213&lt;&gt;F213,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I213" t="inlineStr"/>
     </row>
     <row r="214">
       <c r="A214" s="5" t="n">
@@ -19266,7 +19056,6 @@
         <f>IF(G214&lt;&gt;F214,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I214" t="inlineStr"/>
     </row>
     <row r="215">
       <c r="A215" s="5" t="n">
@@ -19303,7 +19092,6 @@
         <f>IF(G215&lt;&gt;F215,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I215" t="inlineStr"/>
     </row>
     <row r="216">
       <c r="A216" s="5" t="n">
@@ -19340,7 +19128,6 @@
         <f>IF(G216&lt;&gt;F216,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I216" t="inlineStr"/>
     </row>
     <row r="217">
       <c r="A217" s="5" t="n">
@@ -19377,7 +19164,6 @@
         <f>IF(G217&lt;&gt;F217,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I217" t="inlineStr"/>
     </row>
     <row r="218">
       <c r="A218" s="5" t="n">
@@ -19414,7 +19200,6 @@
         <f>IF(G218&lt;&gt;F218,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I218" t="inlineStr"/>
     </row>
     <row r="219">
       <c r="A219" s="5" t="n">
@@ -19451,7 +19236,6 @@
         <f>IF(G219&lt;&gt;F219,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I219" t="inlineStr"/>
     </row>
     <row r="220">
       <c r="A220" s="5" t="n">
@@ -19488,7 +19272,6 @@
         <f>IF(G220&lt;&gt;F220,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I220" t="inlineStr"/>
     </row>
     <row r="221">
       <c r="A221" s="5" t="n">
@@ -19525,7 +19308,6 @@
         <f>IF(G221&lt;&gt;F221,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I221" t="inlineStr"/>
     </row>
     <row r="222">
       <c r="A222" s="5" t="n">
@@ -19562,7 +19344,6 @@
         <f>IF(G222&lt;&gt;F222,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I222" t="inlineStr"/>
     </row>
     <row r="223">
       <c r="A223" s="5" t="n">
@@ -19599,7 +19380,6 @@
         <f>IF(G223&lt;&gt;F223,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I223" t="inlineStr"/>
     </row>
     <row r="224">
       <c r="A224" s="5" t="n">
@@ -19636,7 +19416,6 @@
         <f>IF(G224&lt;&gt;F224,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I224" t="inlineStr"/>
     </row>
     <row r="225">
       <c r="A225" s="5" t="n">
@@ -19673,7 +19452,6 @@
         <f>IF(G225&lt;&gt;F225,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I225" t="inlineStr"/>
     </row>
     <row r="226">
       <c r="A226" s="5" t="n">
@@ -19710,7 +19488,6 @@
         <f>IF(G226&lt;&gt;F226,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I226" t="inlineStr"/>
     </row>
     <row r="227">
       <c r="A227" s="5" t="n">
@@ -19747,7 +19524,6 @@
         <f>IF(G227&lt;&gt;F227,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I227" t="inlineStr"/>
     </row>
     <row r="228">
       <c r="A228" s="5" t="n">
@@ -19784,7 +19560,6 @@
         <f>IF(G228&lt;&gt;F228,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I228" t="inlineStr"/>
     </row>
     <row r="229">
       <c r="A229" s="5" t="n">
@@ -19821,7 +19596,6 @@
         <f>IF(G229&lt;&gt;F229,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I229" t="inlineStr"/>
     </row>
     <row r="230">
       <c r="A230" s="5" t="n">
@@ -19858,7 +19632,6 @@
         <f>IF(G230&lt;&gt;F230,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I230" t="inlineStr"/>
     </row>
     <row r="231">
       <c r="A231" s="5" t="n">
@@ -19895,7 +19668,6 @@
         <f>IF(G231&lt;&gt;F231,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I231" t="inlineStr"/>
     </row>
     <row r="232">
       <c r="A232" s="5" t="n">
@@ -19932,7 +19704,6 @@
         <f>IF(G232&lt;&gt;F232,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I232" t="inlineStr"/>
     </row>
     <row r="233">
       <c r="A233" s="5" t="n">
@@ -19969,7 +19740,6 @@
         <f>IF(G233&lt;&gt;F233,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I233" t="inlineStr"/>
     </row>
     <row r="234">
       <c r="A234" s="5" t="n">
@@ -20006,7 +19776,6 @@
         <f>IF(G234&lt;&gt;F234,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I234" t="inlineStr"/>
     </row>
     <row r="235">
       <c r="A235" s="5" t="n">
@@ -20043,7 +19812,6 @@
         <f>IF(G235&lt;&gt;F235,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I235" t="inlineStr"/>
     </row>
     <row r="236">
       <c r="A236" s="5" t="n">
@@ -20080,7 +19848,6 @@
         <f>IF(G236&lt;&gt;F236,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I236" t="inlineStr"/>
     </row>
     <row r="237">
       <c r="A237" s="5" t="n">
@@ -20117,7 +19884,6 @@
         <f>IF(G237&lt;&gt;F237,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I237" t="inlineStr"/>
     </row>
     <row r="238">
       <c r="A238" s="5" t="n">
@@ -20154,7 +19920,6 @@
         <f>IF(G238&lt;&gt;F238,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I238" t="inlineStr"/>
     </row>
     <row r="239">
       <c r="A239" s="5" t="n">
@@ -20191,7 +19956,6 @@
         <f>IF(G239&lt;&gt;F239,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I239" t="inlineStr"/>
     </row>
     <row r="240">
       <c r="A240" s="5" t="n">
@@ -20228,7 +19992,6 @@
         <f>IF(G240&lt;&gt;F240,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I240" t="inlineStr"/>
     </row>
     <row r="241">
       <c r="A241" s="5" t="n">
@@ -20265,7 +20028,6 @@
         <f>IF(G241&lt;&gt;F241,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I241" t="inlineStr"/>
     </row>
     <row r="242">
       <c r="A242" s="5" t="n">
@@ -20302,7 +20064,6 @@
         <f>IF(G242&lt;&gt;F242,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I242" t="inlineStr"/>
     </row>
     <row r="243">
       <c r="A243" s="5" t="n">
@@ -20339,7 +20100,6 @@
         <f>IF(G243&lt;&gt;F243,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I243" t="inlineStr"/>
     </row>
     <row r="244">
       <c r="A244" s="5" t="n">
@@ -20376,7 +20136,6 @@
         <f>IF(G244&lt;&gt;F244,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I244" t="inlineStr"/>
     </row>
     <row r="245">
       <c r="A245" s="5" t="n">
@@ -20413,7 +20172,6 @@
         <f>IF(G245&lt;&gt;F245,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I245" t="inlineStr"/>
     </row>
     <row r="246">
       <c r="A246" s="5" t="n">
@@ -20450,7 +20208,6 @@
         <f>IF(G246&lt;&gt;F246,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I246" t="inlineStr"/>
     </row>
     <row r="247">
       <c r="A247" s="5" t="n">
@@ -20487,7 +20244,6 @@
         <f>IF(G247&lt;&gt;F247,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I247" t="inlineStr"/>
     </row>
     <row r="248">
       <c r="A248" s="5" t="n">
@@ -20524,7 +20280,6 @@
         <f>IF(G248&lt;&gt;F248,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I248" t="inlineStr"/>
     </row>
     <row r="249">
       <c r="A249" s="5" t="n">
@@ -20561,7 +20316,6 @@
         <f>IF(G249&lt;&gt;F249,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I249" t="inlineStr"/>
     </row>
     <row r="250">
       <c r="A250" s="5" t="n">
@@ -20598,7 +20352,6 @@
         <f>IF(G250&lt;&gt;F250,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I250" t="inlineStr"/>
     </row>
     <row r="251">
       <c r="A251" s="5" t="n">
@@ -20635,7 +20388,6 @@
         <f>IF(G251&lt;&gt;F251,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I251" t="inlineStr"/>
     </row>
     <row r="252">
       <c r="A252" s="5" t="n">
@@ -20672,7 +20424,6 @@
         <f>IF(G252&lt;&gt;F252,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I252" t="inlineStr"/>
     </row>
     <row r="253">
       <c r="A253" s="5" t="n">
@@ -20709,7 +20460,6 @@
         <f>IF(G253&lt;&gt;F253,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I253" t="inlineStr"/>
     </row>
     <row r="254">
       <c r="A254" s="5" t="n">
@@ -20746,7 +20496,6 @@
         <f>IF(G254&lt;&gt;F254,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I254" t="inlineStr"/>
     </row>
     <row r="255">
       <c r="A255" s="5" t="n">
@@ -20783,7 +20532,6 @@
         <f>IF(G255&lt;&gt;F255,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I255" t="inlineStr"/>
     </row>
     <row r="256">
       <c r="A256" s="5" t="n">
@@ -20820,7 +20568,6 @@
         <f>IF(G256&lt;&gt;F256,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I256" t="inlineStr"/>
     </row>
     <row r="257">
       <c r="A257" s="5" t="n">
@@ -20857,7 +20604,6 @@
         <f>IF(G257&lt;&gt;F257,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I257" t="inlineStr"/>
     </row>
     <row r="258">
       <c r="A258" s="5" t="n">
@@ -20894,7 +20640,6 @@
         <f>IF(G258&lt;&gt;F258,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I258" t="inlineStr"/>
     </row>
     <row r="259">
       <c r="A259" s="5" t="n">
@@ -20931,7 +20676,6 @@
         <f>IF(G259&lt;&gt;F259,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I259" t="inlineStr"/>
     </row>
     <row r="260">
       <c r="A260" s="5" t="n">
@@ -20968,7 +20712,6 @@
         <f>IF(G260&lt;&gt;F260,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I260" t="inlineStr"/>
     </row>
     <row r="261">
       <c r="A261" s="5" t="n">
@@ -21005,7 +20748,6 @@
         <f>IF(G261&lt;&gt;F261,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I261" t="inlineStr"/>
     </row>
     <row r="262">
       <c r="A262" s="5" t="n">
@@ -21042,7 +20784,6 @@
         <f>IF(G262&lt;&gt;F262,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I262" t="inlineStr"/>
     </row>
     <row r="263">
       <c r="A263" s="5" t="n">
@@ -21079,7 +20820,6 @@
         <f>IF(G263&lt;&gt;F263,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I263" t="inlineStr"/>
     </row>
     <row r="264">
       <c r="A264" s="5" t="n">
@@ -21116,7 +20856,6 @@
         <f>IF(G264&lt;&gt;F264,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I264" t="inlineStr"/>
     </row>
     <row r="265">
       <c r="A265" s="5" t="n">
@@ -21153,7 +20892,6 @@
         <f>IF(G265&lt;&gt;F265,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I265" t="inlineStr"/>
     </row>
     <row r="266">
       <c r="A266" s="5" t="n">
@@ -21190,7 +20928,6 @@
         <f>IF(G266&lt;&gt;F266,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I266" t="inlineStr"/>
     </row>
     <row r="267">
       <c r="A267" s="5" t="n">
@@ -21227,7 +20964,6 @@
         <f>IF(G267&lt;&gt;F267,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I267" t="inlineStr"/>
     </row>
     <row r="268">
       <c r="A268" s="5" t="n">
@@ -21264,7 +21000,6 @@
         <f>IF(G268&lt;&gt;F268,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I268" t="inlineStr"/>
     </row>
     <row r="269">
       <c r="A269" s="5" t="n">
@@ -21301,7 +21036,6 @@
         <f>IF(G269&lt;&gt;F269,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I269" t="inlineStr"/>
     </row>
     <row r="270">
       <c r="A270" s="5" t="n">
@@ -21338,7 +21072,6 @@
         <f>IF(G270&lt;&gt;F270,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I270" t="inlineStr"/>
     </row>
     <row r="271">
       <c r="A271" s="5" t="n">
@@ -21375,7 +21108,6 @@
         <f>IF(G271&lt;&gt;F271,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I271" t="inlineStr"/>
     </row>
     <row r="272">
       <c r="A272" s="5" t="n">
@@ -21412,7 +21144,6 @@
         <f>IF(G272&lt;&gt;F272,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I272" t="inlineStr"/>
     </row>
     <row r="273">
       <c r="A273" s="5" t="n">
@@ -21449,7 +21180,6 @@
         <f>IF(G273&lt;&gt;F273,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I273" t="inlineStr"/>
     </row>
     <row r="274">
       <c r="A274" s="5" t="n">
@@ -21486,7 +21216,6 @@
         <f>IF(G274&lt;&gt;F274,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I274" t="inlineStr"/>
     </row>
     <row r="275">
       <c r="A275" s="5" t="n">
@@ -21523,7 +21252,6 @@
         <f>IF(G275&lt;&gt;F275,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I275" t="inlineStr"/>
     </row>
     <row r="276">
       <c r="A276" s="5" t="n">
@@ -21560,7 +21288,6 @@
         <f>IF(G276&lt;&gt;F276,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I276" t="inlineStr"/>
     </row>
     <row r="277">
       <c r="A277" s="5" t="n">
@@ -21597,7 +21324,6 @@
         <f>IF(G277&lt;&gt;F277,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I277" t="inlineStr"/>
     </row>
     <row r="278">
       <c r="A278" s="5" t="n">
@@ -21634,7 +21360,6 @@
         <f>IF(G278&lt;&gt;F278,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I278" t="inlineStr"/>
     </row>
     <row r="279">
       <c r="A279" s="5" t="n">
@@ -21671,7 +21396,6 @@
         <f>IF(G279&lt;&gt;F279,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I279" t="inlineStr"/>
     </row>
     <row r="280">
       <c r="A280" s="5" t="n">
@@ -21708,7 +21432,6 @@
         <f>IF(G280&lt;&gt;F280,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I280" t="inlineStr"/>
     </row>
     <row r="281">
       <c r="A281" s="5" t="n">
@@ -21745,7 +21468,6 @@
         <f>IF(G281&lt;&gt;F281,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I281" t="inlineStr"/>
     </row>
     <row r="282">
       <c r="A282" s="5" t="n">
@@ -21782,7 +21504,6 @@
         <f>IF(G282&lt;&gt;F282,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I282" t="inlineStr"/>
     </row>
     <row r="283">
       <c r="A283" s="5" t="n">
@@ -21819,7 +21540,6 @@
         <f>IF(G283&lt;&gt;F283,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I283" t="inlineStr"/>
     </row>
     <row r="284">
       <c r="A284" s="5" t="n">
@@ -21856,7 +21576,6 @@
         <f>IF(G284&lt;&gt;F284,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I284" t="inlineStr"/>
     </row>
     <row r="285">
       <c r="A285" s="5" t="n">
@@ -21893,7 +21612,6 @@
         <f>IF(G285&lt;&gt;F285,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I285" t="inlineStr"/>
     </row>
     <row r="286">
       <c r="A286" s="5" t="n">
@@ -21930,7 +21648,6 @@
         <f>IF(G286&lt;&gt;F286,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I286" t="inlineStr"/>
     </row>
     <row r="287">
       <c r="A287" s="5" t="n">
@@ -21967,7 +21684,6 @@
         <f>IF(G287&lt;&gt;F287,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I287" t="inlineStr"/>
     </row>
     <row r="288">
       <c r="A288" s="5" t="n">
@@ -22004,7 +21720,6 @@
         <f>IF(G288&lt;&gt;F288,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I288" t="inlineStr"/>
     </row>
     <row r="289">
       <c r="A289" s="5" t="n">
@@ -22041,7 +21756,6 @@
         <f>IF(G289&lt;&gt;F289,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I289" t="inlineStr"/>
     </row>
     <row r="290">
       <c r="A290" s="5" t="n">
@@ -22078,7 +21792,6 @@
         <f>IF(G290&lt;&gt;F290,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I290" t="inlineStr"/>
     </row>
     <row r="291">
       <c r="A291" s="5" t="n">
@@ -22115,7 +21828,6 @@
         <f>IF(G291&lt;&gt;F291,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I291" t="inlineStr"/>
     </row>
     <row r="292">
       <c r="A292" s="5" t="n">
@@ -22152,7 +21864,6 @@
         <f>IF(G292&lt;&gt;F292,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I292" t="inlineStr"/>
     </row>
     <row r="293">
       <c r="A293" s="5" t="n">
@@ -22189,7 +21900,6 @@
         <f>IF(G293&lt;&gt;F293,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I293" t="inlineStr"/>
     </row>
     <row r="294">
       <c r="A294" s="5" t="n">
@@ -22226,7 +21936,6 @@
         <f>IF(G294&lt;&gt;F294,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I294" t="inlineStr"/>
     </row>
     <row r="295">
       <c r="A295" s="5" t="n">
@@ -22263,7 +21972,6 @@
         <f>IF(G295&lt;&gt;F295,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I295" t="inlineStr"/>
     </row>
     <row r="296">
       <c r="A296" s="5" t="n">
@@ -22300,7 +22008,6 @@
         <f>IF(G296&lt;&gt;F296,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I296" t="inlineStr"/>
     </row>
     <row r="297">
       <c r="A297" s="5" t="n">
@@ -22337,7 +22044,6 @@
         <f>IF(G297&lt;&gt;F297,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I297" t="inlineStr"/>
     </row>
     <row r="298">
       <c r="A298" s="5" t="n">
@@ -22374,7 +22080,6 @@
         <f>IF(G298&lt;&gt;F298,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I298" t="inlineStr"/>
     </row>
     <row r="299">
       <c r="A299" s="5" t="n">
@@ -22411,7 +22116,6 @@
         <f>IF(G299&lt;&gt;F299,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I299" t="inlineStr"/>
     </row>
     <row r="300">
       <c r="A300" s="5" t="n">
@@ -22448,7 +22152,6 @@
         <f>IF(G300&lt;&gt;F300,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I300" t="inlineStr"/>
     </row>
     <row r="301">
       <c r="A301" s="5" t="n">
@@ -22485,7 +22188,6 @@
         <f>IF(G301&lt;&gt;F301,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I301" t="inlineStr"/>
     </row>
     <row r="302">
       <c r="A302" s="5" t="n">
@@ -22522,7 +22224,6 @@
         <f>IF(G302&lt;&gt;F302,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I302" t="inlineStr"/>
     </row>
     <row r="303">
       <c r="A303" s="5" t="n">
@@ -22559,7 +22260,6 @@
         <f>IF(G303&lt;&gt;F303,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I303" t="inlineStr"/>
     </row>
     <row r="304">
       <c r="A304" s="5" t="n">
@@ -22596,7 +22296,6 @@
         <f>IF(G304&lt;&gt;F304,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I304" t="inlineStr"/>
     </row>
     <row r="305">
       <c r="A305" s="5" t="n">
@@ -22633,7 +22332,6 @@
         <f>IF(G305&lt;&gt;F305,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I305" t="inlineStr"/>
     </row>
     <row r="306">
       <c r="A306" s="5" t="n">
@@ -22670,7 +22368,6 @@
         <f>IF(G306&lt;&gt;F306,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I306" t="inlineStr"/>
     </row>
     <row r="307">
       <c r="A307" s="5" t="n">
@@ -22707,7 +22404,6 @@
         <f>IF(G307&lt;&gt;F307,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I307" t="inlineStr"/>
     </row>
     <row r="308">
       <c r="A308" s="5" t="n">
@@ -22744,7 +22440,6 @@
         <f>IF(G308&lt;&gt;F308,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I308" t="inlineStr"/>
     </row>
     <row r="309">
       <c r="A309" s="5" t="n">
@@ -22781,7 +22476,6 @@
         <f>IF(G309&lt;&gt;F309,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I309" t="inlineStr"/>
     </row>
     <row r="310">
       <c r="A310" s="5" t="n">
@@ -22818,7 +22512,6 @@
         <f>IF(G310&lt;&gt;F310,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I310" t="inlineStr"/>
     </row>
     <row r="311">
       <c r="A311" s="5" t="n">
@@ -22855,7 +22548,6 @@
         <f>IF(G311&lt;&gt;F311,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I311" t="inlineStr"/>
     </row>
     <row r="312">
       <c r="A312" s="5" t="n">
@@ -22892,7 +22584,6 @@
         <f>IF(G312&lt;&gt;F312,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I312" t="inlineStr"/>
     </row>
     <row r="313">
       <c r="A313" s="5" t="n">
@@ -22929,7 +22620,6 @@
         <f>IF(G313&lt;&gt;F313,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I313" t="inlineStr"/>
     </row>
     <row r="314">
       <c r="A314" s="5" t="n">
@@ -22966,7 +22656,6 @@
         <f>IF(G314&lt;&gt;F314,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I314" t="inlineStr"/>
     </row>
     <row r="315">
       <c r="A315" s="5" t="n">
@@ -23003,7 +22692,6 @@
         <f>IF(G315&lt;&gt;F315,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I315" t="inlineStr"/>
     </row>
     <row r="316">
       <c r="A316" s="5" t="n">
@@ -23040,7 +22728,6 @@
         <f>IF(G316&lt;&gt;F316,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I316" t="inlineStr"/>
     </row>
     <row r="317">
       <c r="A317" s="5" t="n">
@@ -23077,7 +22764,6 @@
         <f>IF(G317&lt;&gt;F317,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I317" t="inlineStr"/>
     </row>
     <row r="318">
       <c r="A318" s="5" t="n">
@@ -23114,7 +22800,6 @@
         <f>IF(G318&lt;&gt;F318,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I318" t="inlineStr"/>
     </row>
     <row r="319">
       <c r="A319" s="5" t="n">
@@ -23151,7 +22836,6 @@
         <f>IF(G319&lt;&gt;F319,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I319" t="inlineStr"/>
     </row>
     <row r="320">
       <c r="A320" s="5" t="n">
@@ -23188,7 +22872,6 @@
         <f>IF(G320&lt;&gt;F320,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I320" t="inlineStr"/>
     </row>
     <row r="321">
       <c r="A321" s="5" t="n">
@@ -23225,7 +22908,6 @@
         <f>IF(G321&lt;&gt;F321,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I321" t="inlineStr"/>
     </row>
     <row r="322">
       <c r="A322" s="5" t="n">
@@ -23262,7 +22944,6 @@
         <f>IF(G322&lt;&gt;F322,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I322" t="inlineStr"/>
     </row>
     <row r="323">
       <c r="A323" s="5" t="n">
@@ -23299,7 +22980,6 @@
         <f>IF(G323&lt;&gt;F323,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I323" t="inlineStr"/>
     </row>
     <row r="324">
       <c r="A324" s="5" t="n">
@@ -23336,7 +23016,6 @@
         <f>IF(G324&lt;&gt;F324,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I324" t="inlineStr"/>
     </row>
     <row r="325">
       <c r="A325" s="5" t="n">
@@ -23373,7 +23052,6 @@
         <f>IF(G325&lt;&gt;F325,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I325" t="inlineStr"/>
     </row>
     <row r="326">
       <c r="A326" s="5" t="n">
@@ -23410,7 +23088,6 @@
         <f>IF(G326&lt;&gt;F326,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I326" t="inlineStr"/>
     </row>
     <row r="327">
       <c r="A327" s="5" t="n">
@@ -23447,7 +23124,6 @@
         <f>IF(G327&lt;&gt;F327,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I327" t="inlineStr"/>
     </row>
     <row r="328">
       <c r="A328" s="5" t="n">
@@ -23484,7 +23160,6 @@
         <f>IF(G328&lt;&gt;F328,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I328" t="inlineStr"/>
     </row>
     <row r="329">
       <c r="A329" s="5" t="n">
@@ -23521,7 +23196,6 @@
         <f>IF(G329&lt;&gt;F329,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I329" t="inlineStr"/>
     </row>
     <row r="330">
       <c r="A330" s="5" t="n">
@@ -23558,7 +23232,6 @@
         <f>IF(G330&lt;&gt;F330,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I330" t="inlineStr"/>
     </row>
     <row r="331">
       <c r="A331" s="5" t="n">
@@ -23595,7 +23268,6 @@
         <f>IF(G331&lt;&gt;F331,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I331" t="inlineStr"/>
     </row>
     <row r="332">
       <c r="A332" s="5" t="n">
@@ -23632,7 +23304,6 @@
         <f>IF(G332&lt;&gt;F332,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I332" t="inlineStr"/>
     </row>
     <row r="333">
       <c r="A333" s="5" t="n">
@@ -23669,7 +23340,6 @@
         <f>IF(G333&lt;&gt;F333,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I333" t="inlineStr"/>
     </row>
     <row r="334">
       <c r="A334" s="5" t="n">
@@ -23706,7 +23376,6 @@
         <f>IF(G334&lt;&gt;F334,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I334" t="inlineStr"/>
     </row>
     <row r="335">
       <c r="A335" s="5" t="n">
@@ -23743,7 +23412,6 @@
         <f>IF(G335&lt;&gt;F335,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I335" t="inlineStr"/>
     </row>
     <row r="336">
       <c r="A336" s="5" t="n">
@@ -23780,7 +23448,6 @@
         <f>IF(G336&lt;&gt;F336,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I336" t="inlineStr"/>
     </row>
     <row r="337">
       <c r="A337" s="5" t="n">
@@ -23817,7 +23484,6 @@
         <f>IF(G337&lt;&gt;F337,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I337" t="inlineStr"/>
     </row>
     <row r="338">
       <c r="A338" s="5" t="n">
@@ -23854,7 +23520,6 @@
         <f>IF(G338&lt;&gt;F338,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I338" t="inlineStr"/>
     </row>
     <row r="339">
       <c r="A339" s="5" t="n">
@@ -23891,7 +23556,6 @@
         <f>IF(G339&lt;&gt;F339,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I339" t="inlineStr"/>
     </row>
     <row r="340">
       <c r="A340" s="5" t="n">
@@ -23928,7 +23592,6 @@
         <f>IF(G340&lt;&gt;F340,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I340" t="inlineStr"/>
     </row>
     <row r="341">
       <c r="A341" s="5" t="n">
@@ -23965,7 +23628,6 @@
         <f>IF(G341&lt;&gt;F341,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I341" t="inlineStr"/>
     </row>
     <row r="342">
       <c r="A342" s="5" t="n">
@@ -24002,7 +23664,6 @@
         <f>IF(G342&lt;&gt;F342,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I342" t="inlineStr"/>
     </row>
     <row r="343">
       <c r="A343" s="5" t="n">
@@ -24039,7 +23700,6 @@
         <f>IF(G343&lt;&gt;F343,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I343" t="inlineStr"/>
     </row>
     <row r="344">
       <c r="A344" s="5" t="n">
@@ -24076,7 +23736,6 @@
         <f>IF(G344&lt;&gt;F344,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I344" t="inlineStr"/>
     </row>
     <row r="345">
       <c r="A345" s="5" t="n">
@@ -24113,7 +23772,6 @@
         <f>IF(G345&lt;&gt;F345,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I345" t="inlineStr"/>
     </row>
     <row r="346">
       <c r="A346" s="5" t="n">
@@ -24150,7 +23808,6 @@
         <f>IF(G346&lt;&gt;F346,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I346" t="inlineStr"/>
     </row>
     <row r="347">
       <c r="A347" s="5" t="n">
@@ -24187,7 +23844,6 @@
         <f>IF(G347&lt;&gt;F347,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I347" t="inlineStr"/>
     </row>
     <row r="348">
       <c r="A348" s="5" t="n">
@@ -24224,7 +23880,6 @@
         <f>IF(G348&lt;&gt;F348,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I348" t="inlineStr"/>
     </row>
     <row r="349">
       <c r="A349" s="5" t="n">
@@ -24261,7 +23916,6 @@
         <f>IF(G349&lt;&gt;F349,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I349" t="inlineStr"/>
     </row>
     <row r="350">
       <c r="A350" s="5" t="n">
@@ -24298,7 +23952,6 @@
         <f>IF(G350&lt;&gt;F350,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I350" t="inlineStr"/>
     </row>
     <row r="351">
       <c r="A351" s="5" t="n">
@@ -24335,7 +23988,6 @@
         <f>IF(G351&lt;&gt;F351,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I351" t="inlineStr"/>
     </row>
     <row r="352">
       <c r="A352" s="5" t="n">
@@ -24372,7 +24024,6 @@
         <f>IF(G352&lt;&gt;F352,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I352" t="inlineStr"/>
     </row>
     <row r="353">
       <c r="A353" s="5" t="n">
@@ -24409,7 +24060,6 @@
         <f>IF(G353&lt;&gt;F353,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I353" t="inlineStr"/>
     </row>
     <row r="354">
       <c r="A354" s="5" t="n">
@@ -24446,7 +24096,6 @@
         <f>IF(G354&lt;&gt;F354,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I354" t="inlineStr"/>
     </row>
     <row r="355">
       <c r="A355" s="5" t="n">
@@ -24483,7 +24132,6 @@
         <f>IF(G355&lt;&gt;F355,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I355" t="inlineStr"/>
     </row>
     <row r="356">
       <c r="A356" s="5" t="n">
@@ -24520,7 +24168,6 @@
         <f>IF(G356&lt;&gt;F356,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I356" t="inlineStr"/>
     </row>
     <row r="357">
       <c r="A357" s="5" t="n">
@@ -24557,7 +24204,6 @@
         <f>IF(G357&lt;&gt;F357,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I357" t="inlineStr"/>
     </row>
     <row r="358">
       <c r="A358" s="5" t="n">
@@ -24594,7 +24240,6 @@
         <f>IF(G358&lt;&gt;F358,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I358" t="inlineStr"/>
     </row>
     <row r="359">
       <c r="A359" s="5" t="n">
@@ -24631,7 +24276,6 @@
         <f>IF(G359&lt;&gt;F359,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I359" t="inlineStr"/>
     </row>
     <row r="360">
       <c r="A360" s="5" t="n">
@@ -24668,7 +24312,6 @@
         <f>IF(G360&lt;&gt;F360,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I360" t="inlineStr"/>
     </row>
     <row r="361">
       <c r="A361" s="5" t="n">
@@ -24705,7 +24348,6 @@
         <f>IF(G361&lt;&gt;F361,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I361" t="inlineStr"/>
     </row>
     <row r="362">
       <c r="A362" s="5" t="n">
@@ -24742,7 +24384,6 @@
         <f>IF(G362&lt;&gt;F362,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I362" t="inlineStr"/>
     </row>
     <row r="363">
       <c r="A363" s="5" t="n">
@@ -24779,7 +24420,6 @@
         <f>IF(G363&lt;&gt;F363,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I363" t="inlineStr"/>
     </row>
     <row r="364">
       <c r="A364" s="5" t="n">
@@ -24816,7 +24456,6 @@
         <f>IF(G364&lt;&gt;F364,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I364" t="inlineStr"/>
     </row>
     <row r="365">
       <c r="A365" s="5" t="n">
@@ -24853,7 +24492,6 @@
         <f>IF(G365&lt;&gt;F365,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I365" t="inlineStr"/>
     </row>
     <row r="366">
       <c r="A366" s="5" t="n">
@@ -24890,7 +24528,6 @@
         <f>IF(G366&lt;&gt;F366,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I366" t="inlineStr"/>
     </row>
     <row r="367">
       <c r="A367" s="5" t="n">
@@ -24927,7 +24564,6 @@
         <f>IF(G367&lt;&gt;F367,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I367" t="inlineStr"/>
     </row>
     <row r="368">
       <c r="A368" s="5" t="n">
@@ -24964,7 +24600,6 @@
         <f>IF(G368&lt;&gt;F368,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I368" t="inlineStr"/>
     </row>
     <row r="369">
       <c r="A369" s="5" t="n">
@@ -25001,7 +24636,6 @@
         <f>IF(G369&lt;&gt;F369,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I369" t="inlineStr"/>
     </row>
     <row r="370">
       <c r="A370" s="5" t="n">
@@ -25038,7 +24672,6 @@
         <f>IF(G370&lt;&gt;F370,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I370" t="inlineStr"/>
     </row>
     <row r="371">
       <c r="A371" s="5" t="n">
@@ -25075,7 +24708,6 @@
         <f>IF(G371&lt;&gt;F371,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I371" t="inlineStr"/>
     </row>
     <row r="372">
       <c r="A372" s="5" t="n">
@@ -25112,7 +24744,6 @@
         <f>IF(G372&lt;&gt;F372,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I372" t="inlineStr"/>
     </row>
     <row r="373">
       <c r="A373" s="5" t="n">
@@ -25149,7 +24780,6 @@
         <f>IF(G373&lt;&gt;F373,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I373" t="inlineStr"/>
     </row>
     <row r="374">
       <c r="A374" s="5" t="n">
@@ -25186,7 +24816,6 @@
         <f>IF(G374&lt;&gt;F374,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I374" t="inlineStr"/>
     </row>
     <row r="375">
       <c r="A375" s="5" t="n">
@@ -25223,7 +24852,6 @@
         <f>IF(G375&lt;&gt;F375,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I375" t="inlineStr"/>
     </row>
     <row r="376">
       <c r="A376" s="5" t="n">
@@ -25260,7 +24888,6 @@
         <f>IF(G376&lt;&gt;F376,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I376" t="inlineStr"/>
     </row>
     <row r="377">
       <c r="A377" s="5" t="n">
@@ -25297,7 +24924,6 @@
         <f>IF(G377&lt;&gt;F377,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I377" t="inlineStr"/>
     </row>
     <row r="378">
       <c r="A378" s="5" t="n">
@@ -25334,7 +24960,6 @@
         <f>IF(G378&lt;&gt;F378,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I378" t="inlineStr"/>
     </row>
     <row r="379">
       <c r="A379" s="5" t="n">
@@ -25371,7 +24996,6 @@
         <f>IF(G379&lt;&gt;F379,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I379" t="inlineStr"/>
     </row>
     <row r="380">
       <c r="A380" s="5" t="n">
@@ -25408,7 +25032,6 @@
         <f>IF(G380&lt;&gt;F380,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I380" t="inlineStr"/>
     </row>
     <row r="381">
       <c r="A381" s="5" t="n">
@@ -25445,7 +25068,6 @@
         <f>IF(G381&lt;&gt;F381,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I381" t="inlineStr"/>
     </row>
     <row r="382">
       <c r="A382" s="5" t="n">
@@ -25482,7 +25104,6 @@
         <f>IF(G382&lt;&gt;F382,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I382" t="inlineStr"/>
     </row>
     <row r="383">
       <c r="A383" s="5" t="n">
@@ -25519,7 +25140,6 @@
         <f>IF(G383&lt;&gt;F383,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I383" t="inlineStr"/>
     </row>
     <row r="384">
       <c r="A384" s="5" t="n">
@@ -25556,7 +25176,6 @@
         <f>IF(G384&lt;&gt;F384,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I384" t="inlineStr"/>
     </row>
     <row r="385">
       <c r="A385" s="5" t="n">
@@ -25593,7 +25212,6 @@
         <f>IF(G385&lt;&gt;F385,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I385" t="inlineStr"/>
     </row>
     <row r="386">
       <c r="A386" s="5" t="n">
@@ -25630,7 +25248,6 @@
         <f>IF(G386&lt;&gt;F386,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I386" t="inlineStr"/>
     </row>
     <row r="387">
       <c r="A387" s="5" t="n">
@@ -25667,7 +25284,6 @@
         <f>IF(G387&lt;&gt;F387,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I387" t="inlineStr"/>
     </row>
     <row r="388">
       <c r="A388" s="5" t="n">
@@ -25704,7 +25320,6 @@
         <f>IF(G388&lt;&gt;F388,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I388" t="inlineStr"/>
     </row>
     <row r="389">
       <c r="A389" s="5" t="n">
@@ -25741,7 +25356,6 @@
         <f>IF(G389&lt;&gt;F389,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I389" t="inlineStr"/>
     </row>
     <row r="390">
       <c r="A390" s="5" t="n">
@@ -25778,7 +25392,6 @@
         <f>IF(G390&lt;&gt;F390,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I390" t="inlineStr"/>
     </row>
     <row r="391">
       <c r="A391" s="5" t="n">
@@ -25815,7 +25428,6 @@
         <f>IF(G391&lt;&gt;F391,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I391" t="inlineStr"/>
     </row>
     <row r="392">
       <c r="A392" s="5" t="n">
@@ -25852,7 +25464,6 @@
         <f>IF(G392&lt;&gt;F392,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I392" t="inlineStr"/>
     </row>
     <row r="393">
       <c r="A393" s="5" t="n">
@@ -25889,7 +25500,6 @@
         <f>IF(G393&lt;&gt;F393,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I393" t="inlineStr"/>
     </row>
     <row r="394">
       <c r="A394" s="5" t="n">
@@ -25926,7 +25536,6 @@
         <f>IF(G394&lt;&gt;F394,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I394" t="inlineStr"/>
     </row>
     <row r="395">
       <c r="A395" s="5" t="n">
@@ -25963,7 +25572,6 @@
         <f>IF(G395&lt;&gt;F395,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I395" t="inlineStr"/>
     </row>
     <row r="396">
       <c r="A396" s="5" t="n">
@@ -26000,7 +25608,6 @@
         <f>IF(G396&lt;&gt;F396,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I396" t="inlineStr"/>
     </row>
     <row r="397">
       <c r="A397" s="5" t="n">
@@ -26037,7 +25644,6 @@
         <f>IF(G397&lt;&gt;F397,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I397" t="inlineStr"/>
     </row>
     <row r="398">
       <c r="A398" s="5" t="n">
@@ -26074,7 +25680,6 @@
         <f>IF(G398&lt;&gt;F398,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I398" t="inlineStr"/>
     </row>
     <row r="399">
       <c r="A399" s="5" t="n">
@@ -26111,7 +25716,6 @@
         <f>IF(G399&lt;&gt;F399,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I399" t="inlineStr"/>
     </row>
     <row r="400">
       <c r="A400" s="5" t="n">
@@ -26148,7 +25752,6 @@
         <f>IF(G400&lt;&gt;F400,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I400" t="inlineStr"/>
     </row>
     <row r="401">
       <c r="A401" s="5" t="n">
@@ -26185,7 +25788,6 @@
         <f>IF(G401&lt;&gt;F401,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I401" t="inlineStr"/>
     </row>
     <row r="402">
       <c r="A402" s="5" t="n">
@@ -26222,7 +25824,6 @@
         <f>IF(G402&lt;&gt;F402,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I402" t="inlineStr"/>
     </row>
     <row r="403">
       <c r="A403" s="5" t="n">
@@ -26259,7 +25860,6 @@
         <f>IF(G403&lt;&gt;F403,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I403" t="inlineStr"/>
     </row>
     <row r="404">
       <c r="A404" s="5" t="n">
@@ -26296,7 +25896,6 @@
         <f>IF(G404&lt;&gt;F404,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I404" t="inlineStr"/>
     </row>
     <row r="405">
       <c r="A405" s="5" t="n">
@@ -26333,7 +25932,6 @@
         <f>IF(G405&lt;&gt;F405,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I405" t="inlineStr"/>
     </row>
     <row r="406">
       <c r="A406" s="5" t="n">
@@ -26370,7 +25968,6 @@
         <f>IF(G406&lt;&gt;F406,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I406" t="inlineStr"/>
     </row>
     <row r="407">
       <c r="A407" s="5" t="n">
@@ -26407,7 +26004,6 @@
         <f>IF(G407&lt;&gt;F407,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I407" t="inlineStr"/>
     </row>
     <row r="408">
       <c r="A408" s="5" t="n">
@@ -26444,7 +26040,6 @@
         <f>IF(G408&lt;&gt;F408,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I408" t="inlineStr"/>
     </row>
     <row r="409">
       <c r="A409" s="5" t="n">
@@ -26481,7 +26076,6 @@
         <f>IF(G409&lt;&gt;F409,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I409" t="inlineStr"/>
     </row>
     <row r="410">
       <c r="A410" s="5" t="n">
@@ -26518,7 +26112,6 @@
         <f>IF(G410&lt;&gt;F410,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I410" t="inlineStr"/>
     </row>
     <row r="411">
       <c r="A411" s="5" t="n">
@@ -26555,7 +26148,6 @@
         <f>IF(G411&lt;&gt;F411,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I411" t="inlineStr"/>
     </row>
     <row r="412">
       <c r="A412" s="5" t="n">
@@ -26592,7 +26184,6 @@
         <f>IF(G412&lt;&gt;F412,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I412" t="inlineStr"/>
     </row>
     <row r="413">
       <c r="A413" s="5" t="n">
@@ -26629,7 +26220,6 @@
         <f>IF(G413&lt;&gt;F413,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I413" t="inlineStr"/>
     </row>
     <row r="414">
       <c r="A414" s="5" t="n">
@@ -26666,7 +26256,6 @@
         <f>IF(G414&lt;&gt;F414,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I414" t="inlineStr"/>
     </row>
     <row r="415">
       <c r="A415" s="5" t="n">
@@ -26703,7 +26292,6 @@
         <f>IF(G415&lt;&gt;F415,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I415" t="inlineStr"/>
     </row>
     <row r="416">
       <c r="A416" s="5" t="n">
@@ -26740,7 +26328,6 @@
         <f>IF(G416&lt;&gt;F416,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I416" t="inlineStr"/>
     </row>
     <row r="417">
       <c r="A417" s="5" t="n">
@@ -26777,7 +26364,6 @@
         <f>IF(G417&lt;&gt;F417,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I417" t="inlineStr"/>
     </row>
     <row r="418">
       <c r="A418" s="5" t="n">
@@ -26814,7 +26400,6 @@
         <f>IF(G418&lt;&gt;F418,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I418" t="inlineStr"/>
     </row>
     <row r="419">
       <c r="A419" s="5" t="n">
@@ -26851,7 +26436,6 @@
         <f>IF(G419&lt;&gt;F419,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I419" t="inlineStr"/>
     </row>
     <row r="420">
       <c r="A420" s="5" t="n">
@@ -26888,7 +26472,6 @@
         <f>IF(G420&lt;&gt;F420,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I420" t="inlineStr"/>
     </row>
     <row r="421">
       <c r="A421" s="5" t="n">
@@ -26925,7 +26508,6 @@
         <f>IF(G421&lt;&gt;F421,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I421" t="inlineStr"/>
     </row>
     <row r="422">
       <c r="A422" s="5" t="n">
@@ -26962,7 +26544,6 @@
         <f>IF(G422&lt;&gt;F422,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I422" t="inlineStr"/>
     </row>
     <row r="423">
       <c r="A423" s="5" t="n">
@@ -26999,7 +26580,6 @@
         <f>IF(G423&lt;&gt;F423,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I423" t="inlineStr"/>
     </row>
     <row r="424">
       <c r="A424" s="5" t="n">
@@ -27036,7 +26616,6 @@
         <f>IF(G424&lt;&gt;F424,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I424" t="inlineStr"/>
     </row>
     <row r="425">
       <c r="A425" s="5" t="n">
@@ -27073,7 +26652,6 @@
         <f>IF(G425&lt;&gt;F425,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I425" t="inlineStr"/>
     </row>
     <row r="426">
       <c r="A426" s="5" t="n">
@@ -27110,7 +26688,6 @@
         <f>IF(G426&lt;&gt;F426,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I426" t="inlineStr"/>
     </row>
     <row r="427">
       <c r="A427" s="5" t="n">
@@ -27147,7 +26724,6 @@
         <f>IF(G427&lt;&gt;F427,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I427" t="inlineStr"/>
     </row>
     <row r="428">
       <c r="A428" s="5" t="n">
@@ -27184,7 +26760,6 @@
         <f>IF(G428&lt;&gt;F428,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I428" t="inlineStr"/>
     </row>
     <row r="429">
       <c r="A429" s="5" t="n">
@@ -27221,7 +26796,6 @@
         <f>IF(G429&lt;&gt;F429,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I429" t="inlineStr"/>
     </row>
     <row r="430">
       <c r="A430" s="5" t="n">
@@ -27258,7 +26832,6 @@
         <f>IF(G430&lt;&gt;F430,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I430" t="inlineStr"/>
     </row>
     <row r="431">
       <c r="A431" s="5" t="n">
@@ -27295,7 +26868,6 @@
         <f>IF(G431&lt;&gt;F431,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I431" t="inlineStr"/>
     </row>
     <row r="432">
       <c r="A432" s="5" t="n">
@@ -27332,7 +26904,6 @@
         <f>IF(G432&lt;&gt;F432,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I432" t="inlineStr"/>
     </row>
     <row r="433">
       <c r="A433" s="5" t="n">
@@ -27369,7 +26940,6 @@
         <f>IF(G433&lt;&gt;F433,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I433" t="inlineStr"/>
     </row>
     <row r="434">
       <c r="A434" s="5" t="n">
@@ -27406,7 +26976,6 @@
         <f>IF(G434&lt;&gt;F434,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I434" t="inlineStr"/>
     </row>
     <row r="435">
       <c r="A435" s="5" t="n">
@@ -27443,7 +27012,6 @@
         <f>IF(G435&lt;&gt;F435,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I435" t="inlineStr"/>
     </row>
     <row r="436">
       <c r="A436" s="5" t="n">
@@ -27480,7 +27048,6 @@
         <f>IF(G436&lt;&gt;F436,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I436" t="inlineStr"/>
     </row>
     <row r="437">
       <c r="A437" s="5" t="n">
@@ -27517,7 +27084,6 @@
         <f>IF(G437&lt;&gt;F437,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I437" t="inlineStr"/>
     </row>
     <row r="438">
       <c r="A438" s="5" t="n">
@@ -27554,7 +27120,6 @@
         <f>IF(G438&lt;&gt;F438,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I438" t="inlineStr"/>
     </row>
     <row r="439">
       <c r="A439" s="5" t="n">
@@ -27591,7 +27156,6 @@
         <f>IF(G439&lt;&gt;F439,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I439" t="inlineStr"/>
     </row>
     <row r="440">
       <c r="A440" s="5" t="n">
@@ -27628,7 +27192,6 @@
         <f>IF(G440&lt;&gt;F440,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I440" t="inlineStr"/>
     </row>
     <row r="441">
       <c r="A441" s="5" t="n">
@@ -27665,7 +27228,6 @@
         <f>IF(G441&lt;&gt;F441,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I441" t="inlineStr"/>
     </row>
     <row r="442">
       <c r="A442" s="5" t="n">
@@ -27702,7 +27264,6 @@
         <f>IF(G442&lt;&gt;F442,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I442" t="inlineStr"/>
     </row>
     <row r="443">
       <c r="A443" s="5" t="n">
@@ -27739,7 +27300,6 @@
         <f>IF(G443&lt;&gt;F443,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I443" t="inlineStr"/>
     </row>
     <row r="444">
       <c r="A444" s="5" t="n">
@@ -27776,7 +27336,6 @@
         <f>IF(G444&lt;&gt;F444,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I444" t="inlineStr"/>
     </row>
     <row r="445">
       <c r="A445" s="5" t="n">
@@ -27813,7 +27372,6 @@
         <f>IF(G445&lt;&gt;F445,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I445" t="inlineStr"/>
     </row>
     <row r="446">
       <c r="A446" s="5" t="n">
@@ -27850,7 +27408,6 @@
         <f>IF(G446&lt;&gt;F446,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I446" t="inlineStr"/>
     </row>
     <row r="447">
       <c r="A447" s="5" t="n">
@@ -27887,7 +27444,6 @@
         <f>IF(G447&lt;&gt;F447,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I447" t="inlineStr"/>
     </row>
     <row r="448">
       <c r="A448" s="5" t="n">
@@ -27924,7 +27480,6 @@
         <f>IF(G448&lt;&gt;F448,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I448" t="inlineStr"/>
     </row>
     <row r="449">
       <c r="A449" s="5" t="n">
@@ -27961,7 +27516,6 @@
         <f>IF(G449&lt;&gt;F449,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I449" t="inlineStr"/>
     </row>
     <row r="450">
       <c r="A450" s="5" t="n">
@@ -27998,7 +27552,6 @@
         <f>IF(G450&lt;&gt;F450,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I450" t="inlineStr"/>
     </row>
     <row r="451">
       <c r="A451" s="5" t="n">
@@ -28035,7 +27588,6 @@
         <f>IF(G451&lt;&gt;F451,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I451" t="inlineStr"/>
     </row>
     <row r="452">
       <c r="A452" s="5" t="n">
@@ -28072,7 +27624,6 @@
         <f>IF(G452&lt;&gt;F452,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I452" t="inlineStr"/>
     </row>
     <row r="453">
       <c r="A453" s="5" t="n">
@@ -28109,7 +27660,6 @@
         <f>IF(G453&lt;&gt;F453,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I453" t="inlineStr"/>
     </row>
     <row r="454">
       <c r="A454" s="5" t="n">
@@ -28146,7 +27696,6 @@
         <f>IF(G454&lt;&gt;F454,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I454" t="inlineStr"/>
     </row>
     <row r="455">
       <c r="A455" s="5" t="n">
@@ -28183,7 +27732,6 @@
         <f>IF(G455&lt;&gt;F455,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I455" t="inlineStr"/>
     </row>
     <row r="456">
       <c r="A456" s="5" t="n">
@@ -28220,7 +27768,6 @@
         <f>IF(G456&lt;&gt;F456,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I456" t="inlineStr"/>
     </row>
     <row r="457">
       <c r="A457" s="5" t="n">
@@ -28257,7 +27804,6 @@
         <f>IF(G457&lt;&gt;F457,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I457" t="inlineStr"/>
     </row>
     <row r="458">
       <c r="A458" s="5" t="n">
@@ -28294,7 +27840,6 @@
         <f>IF(G458&lt;&gt;F458,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I458" t="inlineStr"/>
     </row>
     <row r="459">
       <c r="A459" s="5" t="n">
@@ -28331,7 +27876,6 @@
         <f>IF(G459&lt;&gt;F459,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I459" t="inlineStr"/>
     </row>
     <row r="460">
       <c r="A460" s="5" t="n">
@@ -28368,7 +27912,6 @@
         <f>IF(G460&lt;&gt;F460,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I460" t="inlineStr"/>
     </row>
     <row r="461">
       <c r="A461" s="5" t="n">
@@ -28405,7 +27948,6 @@
         <f>IF(G461&lt;&gt;F461,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I461" t="inlineStr"/>
     </row>
     <row r="462">
       <c r="A462" s="5" t="n">
@@ -28442,7 +27984,6 @@
         <f>IF(G462&lt;&gt;F462,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I462" t="inlineStr"/>
     </row>
     <row r="463">
       <c r="A463" s="5" t="n">
@@ -28479,7 +28020,6 @@
         <f>IF(G463&lt;&gt;F463,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I463" t="inlineStr"/>
     </row>
     <row r="464">
       <c r="A464" s="5" t="n">
@@ -28516,7 +28056,6 @@
         <f>IF(G464&lt;&gt;F464,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I464" t="inlineStr"/>
     </row>
     <row r="465">
       <c r="A465" s="5" t="n">
@@ -28553,7 +28092,6 @@
         <f>IF(G465&lt;&gt;F465,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I465" t="inlineStr"/>
     </row>
     <row r="466">
       <c r="A466" s="5" t="n">
@@ -28590,7 +28128,6 @@
         <f>IF(G466&lt;&gt;F466,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I466" t="inlineStr"/>
     </row>
     <row r="467">
       <c r="A467" s="5" t="n">
@@ -28627,7 +28164,6 @@
         <f>IF(G467&lt;&gt;F467,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I467" t="inlineStr"/>
     </row>
     <row r="468">
       <c r="A468" s="5" t="n">
@@ -28664,7 +28200,6 @@
         <f>IF(G468&lt;&gt;F468,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I468" t="inlineStr"/>
     </row>
     <row r="469">
       <c r="A469" s="5" t="n">
@@ -28701,7 +28236,6 @@
         <f>IF(G469&lt;&gt;F469,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I469" t="inlineStr"/>
     </row>
     <row r="470">
       <c r="A470" s="5" t="n">
@@ -28738,7 +28272,6 @@
         <f>IF(G470&lt;&gt;F470,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I470" t="inlineStr"/>
     </row>
     <row r="471">
       <c r="A471" s="5" t="n">
@@ -28775,7 +28308,6 @@
         <f>IF(G471&lt;&gt;F471,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I471" t="inlineStr"/>
     </row>
     <row r="472">
       <c r="A472" s="5" t="n">
@@ -28812,7 +28344,6 @@
         <f>IF(G472&lt;&gt;F472,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I472" t="inlineStr"/>
     </row>
     <row r="473">
       <c r="A473" s="5" t="n">
@@ -28849,7 +28380,6 @@
         <f>IF(G473&lt;&gt;F473,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I473" t="inlineStr"/>
     </row>
     <row r="474">
       <c r="A474" s="5" t="n">
@@ -28886,7 +28416,6 @@
         <f>IF(G474&lt;&gt;F474,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I474" t="inlineStr"/>
     </row>
     <row r="475">
       <c r="A475" s="5" t="n">
@@ -28923,7 +28452,6 @@
         <f>IF(G475&lt;&gt;F475,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I475" t="inlineStr"/>
     </row>
     <row r="476">
       <c r="A476" s="5" t="n">
@@ -28960,7 +28488,6 @@
         <f>IF(G476&lt;&gt;F476,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I476" t="inlineStr"/>
     </row>
     <row r="477">
       <c r="A477" s="5" t="n">
@@ -28997,7 +28524,6 @@
         <f>IF(G477&lt;&gt;F477,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I477" t="inlineStr"/>
     </row>
     <row r="478">
       <c r="A478" s="5" t="n">
@@ -29034,7 +28560,6 @@
         <f>IF(G478&lt;&gt;F478,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I478" t="inlineStr"/>
     </row>
     <row r="479">
       <c r="A479" s="5" t="n">
@@ -29071,7 +28596,6 @@
         <f>IF(G479&lt;&gt;F479,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I479" t="inlineStr"/>
     </row>
     <row r="480">
       <c r="A480" s="5" t="n">
@@ -29108,7 +28632,6 @@
         <f>IF(G480&lt;&gt;F480,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I480" t="inlineStr"/>
     </row>
     <row r="481">
       <c r="A481" s="5" t="n">
@@ -29145,7 +28668,6 @@
         <f>IF(G481&lt;&gt;F481,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I481" t="inlineStr"/>
     </row>
     <row r="482">
       <c r="A482" s="5" t="n">
@@ -29182,7 +28704,6 @@
         <f>IF(G482&lt;&gt;F482,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I482" t="inlineStr"/>
     </row>
     <row r="483">
       <c r="A483" s="5" t="n">
@@ -29219,7 +28740,6 @@
         <f>IF(G483&lt;&gt;F483,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I483" t="inlineStr"/>
     </row>
     <row r="484">
       <c r="A484" s="5" t="n">
@@ -29256,7 +28776,6 @@
         <f>IF(G484&lt;&gt;F484,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I484" t="inlineStr"/>
     </row>
     <row r="485">
       <c r="A485" s="5" t="n">
@@ -29293,7 +28812,6 @@
         <f>IF(G485&lt;&gt;F485,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I485" t="inlineStr"/>
     </row>
     <row r="486">
       <c r="A486" s="5" t="n">
@@ -29330,7 +28848,6 @@
         <f>IF(G486&lt;&gt;F486,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I486" t="inlineStr"/>
     </row>
     <row r="487">
       <c r="A487" s="5" t="n">
@@ -29367,7 +28884,6 @@
         <f>IF(G487&lt;&gt;F487,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I487" t="inlineStr"/>
     </row>
     <row r="488">
       <c r="A488" s="5" t="n">
@@ -29404,7 +28920,6 @@
         <f>IF(G488&lt;&gt;F488,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I488" t="inlineStr"/>
     </row>
     <row r="489">
       <c r="A489" s="5" t="n">
@@ -29441,7 +28956,6 @@
         <f>IF(G489&lt;&gt;F489,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I489" t="inlineStr"/>
     </row>
     <row r="490">
       <c r="A490" s="5" t="n">
@@ -29478,7 +28992,6 @@
         <f>IF(G490&lt;&gt;F490,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I490" t="inlineStr"/>
     </row>
     <row r="491">
       <c r="A491" s="5" t="n">
@@ -29515,7 +29028,6 @@
         <f>IF(G491&lt;&gt;F491,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I491" t="inlineStr"/>
     </row>
     <row r="492">
       <c r="A492" s="5" t="n">
@@ -29552,7 +29064,6 @@
         <f>IF(G492&lt;&gt;F492,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I492" t="inlineStr"/>
     </row>
     <row r="493">
       <c r="A493" s="5" t="n">
@@ -29589,7 +29100,6 @@
         <f>IF(G493&lt;&gt;F493,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I493" t="inlineStr"/>
     </row>
     <row r="494">
       <c r="A494" s="5" t="n">
@@ -29626,7 +29136,6 @@
         <f>IF(G494&lt;&gt;F494,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I494" t="inlineStr"/>
     </row>
     <row r="495">
       <c r="A495" s="5" t="n">
@@ -29663,7 +29172,6 @@
         <f>IF(G495&lt;&gt;F495,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I495" t="inlineStr"/>
     </row>
     <row r="496">
       <c r="A496" s="5" t="n">
@@ -29700,7 +29208,6 @@
         <f>IF(G496&lt;&gt;F496,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I496" t="inlineStr"/>
     </row>
     <row r="497">
       <c r="A497" s="5" t="n">
@@ -29737,7 +29244,6 @@
         <f>IF(G497&lt;&gt;F497,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I497" t="inlineStr"/>
     </row>
     <row r="498">
       <c r="A498" s="5" t="n">
@@ -29774,7 +29280,6 @@
         <f>IF(G498&lt;&gt;F498,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I498" t="inlineStr"/>
     </row>
     <row r="499">
       <c r="A499" s="5" t="n">
@@ -29811,7 +29316,6 @@
         <f>IF(G499&lt;&gt;F499,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I499" t="inlineStr"/>
     </row>
     <row r="500">
       <c r="A500" s="5" t="n">
@@ -29848,7 +29352,6 @@
         <f>IF(G500&lt;&gt;F500,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I500" t="inlineStr"/>
     </row>
     <row r="501">
       <c r="A501" s="5" t="n">
@@ -29885,7 +29388,6 @@
         <f>IF(G501&lt;&gt;F501,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I501" t="inlineStr"/>
     </row>
     <row r="502">
       <c r="A502" s="5" t="n">
@@ -29922,7 +29424,6 @@
         <f>IF(G502&lt;&gt;F502,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I502" t="inlineStr"/>
     </row>
     <row r="503">
       <c r="A503" s="5" t="n">
@@ -29959,7 +29460,6 @@
         <f>IF(G503&lt;&gt;F503,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I503" t="inlineStr"/>
     </row>
     <row r="504">
       <c r="A504" s="5" t="n">
@@ -29996,7 +29496,6 @@
         <f>IF(G504&lt;&gt;F504,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I504" t="inlineStr"/>
     </row>
     <row r="505">
       <c r="A505" s="5" t="n">
@@ -30033,7 +29532,6 @@
         <f>IF(G505&lt;&gt;F505,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I505" t="inlineStr"/>
     </row>
     <row r="506">
       <c r="A506" s="5" t="n">
@@ -30070,7 +29568,6 @@
         <f>IF(G506&lt;&gt;F506,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I506" t="inlineStr"/>
     </row>
     <row r="507">
       <c r="A507" s="5" t="n">
@@ -30107,7 +29604,6 @@
         <f>IF(G507&lt;&gt;F507,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I507" t="inlineStr"/>
     </row>
     <row r="508">
       <c r="A508" s="5" t="n">
@@ -30144,7 +29640,6 @@
         <f>IF(G508&lt;&gt;F508,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I508" t="inlineStr"/>
     </row>
     <row r="509">
       <c r="A509" s="5" t="n">
@@ -30181,7 +29676,6 @@
         <f>IF(G509&lt;&gt;F509,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I509" t="inlineStr"/>
     </row>
     <row r="510">
       <c r="A510" s="5" t="n">
@@ -30218,7 +29712,6 @@
         <f>IF(G510&lt;&gt;F510,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I510" t="inlineStr"/>
     </row>
     <row r="511">
       <c r="A511" s="5" t="n">
@@ -30255,7 +29748,6 @@
         <f>IF(G511&lt;&gt;F511,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I511" t="inlineStr"/>
     </row>
     <row r="512">
       <c r="A512" s="5" t="n">
@@ -30292,7 +29784,6 @@
         <f>IF(G512&lt;&gt;F512,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I512" t="inlineStr"/>
     </row>
     <row r="513">
       <c r="A513" s="5" t="n">
@@ -30329,7 +29820,6 @@
         <f>IF(G513&lt;&gt;F513,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I513" t="inlineStr"/>
     </row>
     <row r="514">
       <c r="A514" s="5" t="n">
@@ -30366,7 +29856,6 @@
         <f>IF(G514&lt;&gt;F514,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I514" t="inlineStr"/>
     </row>
     <row r="515">
       <c r="A515" s="5" t="n">
@@ -30403,7 +29892,6 @@
         <f>IF(G515&lt;&gt;F515,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I515" t="inlineStr"/>
     </row>
     <row r="516">
       <c r="A516" s="5" t="n">
@@ -30440,7 +29928,6 @@
         <f>IF(G516&lt;&gt;F516,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I516" t="inlineStr"/>
     </row>
     <row r="517">
       <c r="A517" s="5" t="n">
@@ -30477,7 +29964,6 @@
         <f>IF(G517&lt;&gt;F517,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I517" t="inlineStr"/>
     </row>
     <row r="518">
       <c r="A518" s="5" t="n">
@@ -30514,7 +30000,6 @@
         <f>IF(G518&lt;&gt;F518,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I518" t="inlineStr"/>
     </row>
     <row r="519">
       <c r="A519" s="5" t="n">
@@ -30551,7 +30036,6 @@
         <f>IF(G519&lt;&gt;F519,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I519" t="inlineStr"/>
     </row>
     <row r="520">
       <c r="A520" s="5" t="n">
@@ -30588,7 +30072,6 @@
         <f>IF(G520&lt;&gt;F520,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I520" t="inlineStr"/>
     </row>
     <row r="521">
       <c r="A521" s="5" t="n">
@@ -30625,7 +30108,6 @@
         <f>IF(G521&lt;&gt;F521,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I521" t="inlineStr"/>
     </row>
     <row r="522">
       <c r="A522" s="5" t="n">
@@ -30662,7 +30144,6 @@
         <f>IF(G522&lt;&gt;F522,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I522" t="inlineStr"/>
     </row>
     <row r="523">
       <c r="A523" s="5" t="n">
@@ -30699,7 +30180,6 @@
         <f>IF(G523&lt;&gt;F523,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I523" t="inlineStr"/>
     </row>
     <row r="524">
       <c r="A524" s="5" t="n">
@@ -30736,7 +30216,6 @@
         <f>IF(G524&lt;&gt;F524,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I524" t="inlineStr"/>
     </row>
     <row r="525">
       <c r="A525" s="5" t="n">
@@ -30773,7 +30252,6 @@
         <f>IF(G525&lt;&gt;F525,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I525" t="inlineStr"/>
     </row>
     <row r="526">
       <c r="A526" s="5" t="n">
@@ -30810,7 +30288,6 @@
         <f>IF(G526&lt;&gt;F526,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I526" t="inlineStr"/>
     </row>
     <row r="527">
       <c r="A527" s="5" t="n">
@@ -30847,7 +30324,6 @@
         <f>IF(G527&lt;&gt;F527,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I527" t="inlineStr"/>
     </row>
     <row r="528">
       <c r="A528" s="5" t="n">
@@ -30884,7 +30360,6 @@
         <f>IF(G528&lt;&gt;F528,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I528" t="inlineStr"/>
     </row>
     <row r="529">
       <c r="A529" s="5" t="n">
@@ -30921,7 +30396,6 @@
         <f>IF(G529&lt;&gt;F529,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I529" t="inlineStr"/>
     </row>
     <row r="530">
       <c r="A530" s="5" t="n">
@@ -30958,7 +30432,6 @@
         <f>IF(G530&lt;&gt;F530,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I530" t="inlineStr"/>
     </row>
     <row r="531">
       <c r="A531" s="5" t="n">
@@ -30995,7 +30468,6 @@
         <f>IF(G531&lt;&gt;F531,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I531" t="inlineStr"/>
     </row>
     <row r="532">
       <c r="A532" s="5" t="n">
@@ -31032,7 +30504,6 @@
         <f>IF(G532&lt;&gt;F532,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I532" t="inlineStr"/>
     </row>
     <row r="533">
       <c r="A533" s="5" t="n">
@@ -31069,7 +30540,6 @@
         <f>IF(G533&lt;&gt;F533,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I533" t="inlineStr"/>
     </row>
     <row r="534">
       <c r="A534" s="5" t="n">
@@ -31106,7 +30576,6 @@
         <f>IF(G534&lt;&gt;F534,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I534" t="inlineStr"/>
     </row>
     <row r="535">
       <c r="A535" s="5" t="n">
@@ -31143,7 +30612,6 @@
         <f>IF(G535&lt;&gt;F535,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I535" t="inlineStr"/>
     </row>
     <row r="536">
       <c r="A536" s="5" t="n">
@@ -31180,7 +30648,6 @@
         <f>IF(G536&lt;&gt;F536,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I536" t="inlineStr"/>
     </row>
     <row r="537">
       <c r="A537" s="5" t="n">
@@ -31217,7 +30684,6 @@
         <f>IF(G537&lt;&gt;F537,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I537" t="inlineStr"/>
     </row>
     <row r="538">
       <c r="A538" s="5" t="n">
@@ -31254,7 +30720,6 @@
         <f>IF(G538&lt;&gt;F538,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I538" t="inlineStr"/>
     </row>
     <row r="539">
       <c r="A539" s="5" t="n">
@@ -31291,7 +30756,6 @@
         <f>IF(G539&lt;&gt;F539,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I539" t="inlineStr"/>
     </row>
     <row r="540">
       <c r="A540" s="5" t="n">
@@ -31328,7 +30792,6 @@
         <f>IF(G540&lt;&gt;F540,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I540" t="inlineStr"/>
     </row>
     <row r="541">
       <c r="A541" s="5" t="n">
@@ -31365,7 +30828,6 @@
         <f>IF(G541&lt;&gt;F541,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I541" t="inlineStr"/>
     </row>
     <row r="542">
       <c r="A542" s="5" t="n">
@@ -31402,7 +30864,6 @@
         <f>IF(G542&lt;&gt;F542,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I542" t="inlineStr"/>
     </row>
     <row r="543">
       <c r="A543" s="5" t="n">
@@ -31439,7 +30900,6 @@
         <f>IF(G543&lt;&gt;F543,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I543" t="inlineStr"/>
     </row>
     <row r="544">
       <c r="A544" s="5" t="n">
@@ -31476,7 +30936,6 @@
         <f>IF(G544&lt;&gt;F544,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I544" t="inlineStr"/>
     </row>
     <row r="545">
       <c r="A545" s="5" t="n">
@@ -31513,7 +30972,6 @@
         <f>IF(G545&lt;&gt;F545,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I545" t="inlineStr"/>
     </row>
     <row r="546">
       <c r="A546" s="5" t="n">
@@ -31550,7 +31008,6 @@
         <f>IF(G546&lt;&gt;F546,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I546" t="inlineStr"/>
     </row>
     <row r="547">
       <c r="A547" s="5" t="n">
@@ -31587,7 +31044,6 @@
         <f>IF(G547&lt;&gt;F547,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I547" t="inlineStr"/>
     </row>
     <row r="548">
       <c r="A548" s="5" t="n">
@@ -31624,7 +31080,6 @@
         <f>IF(G548&lt;&gt;F548,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I548" t="inlineStr"/>
     </row>
     <row r="549">
       <c r="A549" s="5" t="n">
@@ -31661,7 +31116,6 @@
         <f>IF(G549&lt;&gt;F549,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I549" t="inlineStr"/>
     </row>
     <row r="550">
       <c r="A550" s="5" t="n">
@@ -31698,7 +31152,6 @@
         <f>IF(G550&lt;&gt;F550,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I550" t="inlineStr"/>
     </row>
     <row r="551">
       <c r="A551" s="5" t="n">
@@ -31735,7 +31188,6 @@
         <f>IF(G551&lt;&gt;F551,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I551" t="inlineStr"/>
     </row>
     <row r="552">
       <c r="A552" s="5" t="n">
@@ -31772,7 +31224,6 @@
         <f>IF(G552&lt;&gt;F552,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I552" t="inlineStr"/>
     </row>
     <row r="553">
       <c r="A553" s="5" t="n">
@@ -31809,7 +31260,6 @@
         <f>IF(G553&lt;&gt;F553,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I553" t="inlineStr"/>
     </row>
     <row r="554">
       <c r="A554" s="5" t="n">
@@ -31846,7 +31296,6 @@
         <f>IF(G554&lt;&gt;F554,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I554" t="inlineStr"/>
     </row>
     <row r="555">
       <c r="A555" s="5" t="n">
@@ -31883,7 +31332,6 @@
         <f>IF(G555&lt;&gt;F555,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I555" t="inlineStr"/>
     </row>
     <row r="556">
       <c r="A556" s="5" t="n">
@@ -31920,7 +31368,6 @@
         <f>IF(G556&lt;&gt;F556,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I556" t="inlineStr"/>
     </row>
     <row r="557">
       <c r="A557" s="5" t="n">
@@ -31957,7 +31404,6 @@
         <f>IF(G557&lt;&gt;F557,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I557" t="inlineStr"/>
     </row>
     <row r="558">
       <c r="A558" s="5" t="n">
@@ -31994,7 +31440,6 @@
         <f>IF(G558&lt;&gt;F558,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I558" t="inlineStr"/>
     </row>
     <row r="559">
       <c r="A559" s="5" t="n">
@@ -32031,7 +31476,6 @@
         <f>IF(G559&lt;&gt;F559,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I559" t="inlineStr"/>
     </row>
     <row r="560">
       <c r="A560" s="5" t="n">
@@ -32068,7 +31512,6 @@
         <f>IF(G560&lt;&gt;F560,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I560" t="inlineStr"/>
     </row>
     <row r="561">
       <c r="A561" s="5" t="n">
@@ -32105,7 +31548,6 @@
         <f>IF(G561&lt;&gt;F561,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I561" t="inlineStr"/>
     </row>
     <row r="562">
       <c r="A562" s="5" t="n">
@@ -32142,7 +31584,6 @@
         <f>IF(G562&lt;&gt;F562,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I562" t="inlineStr"/>
     </row>
     <row r="563">
       <c r="A563" s="5" t="n">
@@ -32179,7 +31620,6 @@
         <f>IF(G563&lt;&gt;F563,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I563" t="inlineStr"/>
     </row>
     <row r="564">
       <c r="A564" s="5" t="n">
@@ -32216,7 +31656,6 @@
         <f>IF(G564&lt;&gt;F564,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I564" t="inlineStr"/>
     </row>
     <row r="565">
       <c r="A565" s="5" t="n">
@@ -32253,7 +31692,6 @@
         <f>IF(G565&lt;&gt;F565,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I565" t="inlineStr"/>
     </row>
     <row r="566">
       <c r="A566" s="5" t="n">
@@ -32290,7 +31728,6 @@
         <f>IF(G566&lt;&gt;F566,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I566" t="inlineStr"/>
     </row>
     <row r="567">
       <c r="A567" s="5" t="n">
@@ -32327,7 +31764,6 @@
         <f>IF(G567&lt;&gt;F567,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I567" t="inlineStr"/>
     </row>
     <row r="568">
       <c r="A568" s="5" t="n">
@@ -32364,7 +31800,6 @@
         <f>IF(G568&lt;&gt;F568,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I568" t="inlineStr"/>
     </row>
     <row r="569">
       <c r="A569" s="5" t="n">
@@ -32401,7 +31836,6 @@
         <f>IF(G569&lt;&gt;F569,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I569" t="inlineStr"/>
     </row>
     <row r="570">
       <c r="A570" s="5" t="n">
@@ -32438,7 +31872,6 @@
         <f>IF(G570&lt;&gt;F570,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I570" t="inlineStr"/>
     </row>
     <row r="571">
       <c r="A571" s="5" t="n">
@@ -32475,7 +31908,6 @@
         <f>IF(G571&lt;&gt;F571,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I571" t="inlineStr"/>
     </row>
     <row r="572">
       <c r="A572" s="5" t="n">
@@ -32512,7 +31944,6 @@
         <f>IF(G572&lt;&gt;F572,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I572" t="inlineStr"/>
     </row>
     <row r="573">
       <c r="A573" s="5" t="n">
@@ -32549,7 +31980,6 @@
         <f>IF(G573&lt;&gt;F573,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I573" t="inlineStr"/>
     </row>
     <row r="574">
       <c r="A574" s="5" t="n">
@@ -32586,7 +32016,6 @@
         <f>IF(G574&lt;&gt;F574,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I574" t="inlineStr"/>
     </row>
     <row r="575">
       <c r="A575" s="5" t="n">
@@ -32623,7 +32052,6 @@
         <f>IF(G575&lt;&gt;F575,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I575" t="inlineStr"/>
     </row>
     <row r="576">
       <c r="A576" s="5" t="n">
@@ -32660,7 +32088,6 @@
         <f>IF(G576&lt;&gt;F576,"YES","NO")</f>
         <v/>
       </c>
-      <c r="I576" t="inlineStr"/>
     </row>
   </sheetData>
   <conditionalFormatting sqref="A2:I2">
@@ -35569,15 +34996,11 @@
     <row r="1">
       <c r="A1" s="7" t="inlineStr">
         <is>
-          <t>ALL PRO METRO EAST CONSTRUCTION LLC - Profit &amp; Loss 2025</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr"/>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr"/>
-      <c r="B2" t="inlineStr"/>
-    </row>
+          <t>AllPro Construction &amp; Landscape - Profit &amp; Loss 2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
@@ -36041,6 +35464,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="6" t="inlineStr">
         <is>
@@ -36048,6 +35472,7 @@
         </is>
       </c>
     </row>
+    <row r="4"/>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
@@ -36070,6 +35495,7 @@
         <v/>
       </c>
     </row>
+    <row r="7"/>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
         <is>
@@ -36746,6 +36172,7 @@
         <v/>
       </c>
     </row>
+    <row r="15"/>
     <row r="16">
       <c r="A16" s="8" t="inlineStr">
         <is>

</xml_diff>